<commit_message>
Add Final-Form Muzan, Gyokko, and Sabito & Makomo
Final-Form Muzan is a second version of Muzan that gets back up once
(Seven Hearts). Gyokko traps an enemy in his pot. Sabito & Makomo train an
ally for +2 PWR and count as Urokodaki's pupils. Kokushibo trimmed to 50 HP
so Yoriichi stays the strongest.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -11,7 +11,7 @@
     <sheet name="HP % Calculator" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S53"/>
+  <dimension ref="A1:S56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="15" min="1" max="1"/>
@@ -821,12 +821,12 @@
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
-          <t>Muzan Kibutsuji</t>
+          <t>Muzan Kibutsuji (Final Form)</t>
         </is>
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Final Form</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
@@ -836,14 +836,14 @@
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Demon King</t>
+          <t>Demon King · Final Form</t>
         </is>
       </c>
       <c r="E4" s="20" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" s="20" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G4" s="20" t="n">
         <v>17</v>
@@ -855,7 +855,7 @@
         <v>8</v>
       </c>
       <c r="J4" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4" s="21">
         <f>1/F4</f>
@@ -875,23 +875,27 @@
       </c>
       <c r="P4" s="19" t="inlineStr">
         <is>
-          <t>Blood Whips</t>
+          <t>Thorned Flesh Whips</t>
         </is>
       </c>
       <c r="Q4" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−4, and Muzan heals 2 for each enemy hit.</t>
+          <t>Every enemy takes PWR−3, and he heals 3 for each enemy hit.</t>
         </is>
       </c>
       <c r="R4" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S4" s="22" t="n"/>
+      <c r="S4" s="22" t="inlineStr">
+        <is>
+          <t>Seven Hearts: the first time he falls, he gets back up with 20% health.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="26.85" customHeight="1" s="16">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Kokushibo</t>
+          <t>Muzan Kibutsuji</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
@@ -906,14 +910,14 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 1</t>
+          <t>Demon King</t>
         </is>
       </c>
       <c r="E5" s="20" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G5" s="20" t="n">
         <v>17</v>
@@ -925,7 +929,7 @@
         <v>8</v>
       </c>
       <c r="J5" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5" s="21">
         <f>1/F5</f>
@@ -945,12 +949,12 @@
       </c>
       <c r="P5" s="19" t="inlineStr">
         <is>
-          <t>Moon Breathing</t>
+          <t>Blood Whips</t>
         </is>
       </c>
       <c r="Q5" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−4, ignores DEF.</t>
+          <t>Every enemy takes PWR−4, and Muzan heals 2 for each enemy hit.</t>
         </is>
       </c>
       <c r="R5" s="20" t="n">
@@ -961,7 +965,7 @@
     <row r="6" ht="15" customHeight="1" s="16">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Akaza</t>
+          <t>Kokushibo</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
@@ -976,26 +980,26 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 3</t>
+          <t>Upper Moon 1</t>
         </is>
       </c>
       <c r="E6" s="20" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I6" s="20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J6" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="21">
         <f>1/F6</f>
@@ -1015,12 +1019,12 @@
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>Destructive Death</t>
+          <t>Moon Breathing</t>
         </is>
       </c>
       <c r="Q6" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+6.</t>
+          <t>Every enemy takes PWR−4, ignores DEF.</t>
         </is>
       </c>
       <c r="R6" s="20" t="n">
@@ -1031,7 +1035,7 @@
     <row r="7" ht="15" customHeight="1" s="16">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Hantengu</t>
+          <t>Akaza</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
@@ -1046,26 +1050,26 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 4</t>
+          <t>Upper Moon 3</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
         <v>9</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="21">
         <f>1/F7</f>
@@ -1085,27 +1089,23 @@
       </c>
       <c r="P7" s="19" t="inlineStr">
         <is>
-          <t>Cowering Hide</t>
+          <t>Destructive Death</t>
         </is>
       </c>
       <c r="Q7" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
+          <t>Strike for PWR+6.</t>
         </is>
       </c>
       <c r="R7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S7" s="22" t="inlineStr">
-        <is>
-          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
-        </is>
-      </c>
+      <c r="S7" s="22" t="n"/>
     </row>
     <row r="8" ht="26.85" customHeight="1" s="16">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>Doma</t>
+          <t>Hantengu</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
@@ -1120,26 +1120,26 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 2</t>
+          <t>Upper Moon 4</t>
         </is>
       </c>
       <c r="E8" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" s="20" t="n">
         <v>8</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>37</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>11</v>
       </c>
       <c r="H8" s="20" t="n">
         <v>9</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="21">
         <f>1/F8</f>
@@ -1159,23 +1159,27 @@
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Frozen Lotus</t>
+          <t>Cowering Hide</t>
         </is>
       </c>
       <c r="Q8" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 8, ignores DEF.</t>
+          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
         </is>
       </c>
       <c r="R8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S8" s="22" t="n"/>
+      <c r="S8" s="22" t="inlineStr">
+        <is>
+          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="16">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Gyutaro &amp; Daki</t>
+          <t>Doma</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -1190,23 +1194,23 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6</t>
+          <t>Upper Moon 2</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G9" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="H9" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="H9" s="20" t="n">
-        <v>8</v>
-      </c>
       <c r="I9" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" s="20" t="n">
         <v>2</v>
@@ -1229,12 +1233,12 @@
       </c>
       <c r="P9" s="19" t="inlineStr">
         <is>
-          <t>Flying Blood Sickles</t>
+          <t>Frozen Lotus</t>
         </is>
       </c>
       <c r="Q9" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
+          <t>Every enemy takes 8, ignores DEF.</t>
         </is>
       </c>
       <c r="R9" s="20" t="n">
@@ -1245,7 +1249,7 @@
     <row r="10" ht="15" customHeight="1" s="16">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>Kaigaku</t>
+          <t>Gyokko</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -1260,26 +1264,26 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6 · fallen Thunder</t>
+          <t>Upper Moon 5</t>
         </is>
       </c>
       <c r="E10" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J10" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="21">
         <f>1/F10</f>
@@ -1299,27 +1303,23 @@
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>Black Thunder</t>
+          <t>Water Prison Pot</t>
         </is>
       </c>
       <c r="Q10" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3, and a second random enemy takes 4.</t>
+          <t>Traps one enemy: it takes PWR−2 (ignores DEF) and can't act next round.</t>
         </is>
       </c>
       <c r="R10" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S10" s="22" t="inlineStr">
-        <is>
-          <t>Rival: an enemy Zenitsu gets +2 PWR against him.</t>
-        </is>
-      </c>
+      <c r="S10" s="22" t="n"/>
     </row>
     <row r="11" ht="26.85" customHeight="1" s="16">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Enmu</t>
+          <t>Gyutaro &amp; Daki</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
@@ -1334,26 +1334,26 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 1</t>
+          <t>Upper Moon 6</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I11" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J11" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" s="21">
         <f>1/F11</f>
@@ -1373,12 +1373,12 @@
       </c>
       <c r="P11" s="19" t="inlineStr">
         <is>
-          <t>Forced Sleep</t>
+          <t>Flying Blood Sickles</t>
         </is>
       </c>
       <c r="Q11" s="22" t="inlineStr">
         <is>
-          <t>Every enemy has to wait 2 more rounds for their special.</t>
+          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
         </is>
       </c>
       <c r="R11" s="20" t="n">
@@ -1389,7 +1389,7 @@
     <row r="12" ht="15" customHeight="1" s="16">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>Rui</t>
+          <t>Kaigaku</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
@@ -1404,23 +1404,23 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 5</t>
+          <t>Upper Moon 6 · fallen Thunder</t>
         </is>
       </c>
       <c r="E12" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="20" t="n">
         <v>1</v>
@@ -1443,23 +1443,27 @@
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>Cutting Thread Cage</t>
+          <t>Black Thunder</t>
         </is>
       </c>
       <c r="Q12" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR and stun the target next round.</t>
+          <t>Strike for PWR+3, and a second random enemy takes 4.</t>
         </is>
       </c>
       <c r="R12" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S12" s="22" t="n"/>
+      <c r="S12" s="22" t="inlineStr">
+        <is>
+          <t>Rival: an enemy Zenitsu gets +2 PWR against him.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26.85" customHeight="1" s="16">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Kyogai</t>
+          <t>Enmu</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -1474,20 +1478,20 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Former Lower Moon</t>
+          <t>Lower Moon 1</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G13" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I13" s="20" t="n">
         <v>3</v>
@@ -1513,23 +1517,23 @@
       </c>
       <c r="P13" s="19" t="inlineStr">
         <is>
-          <t>Drum Room Spin</t>
+          <t>Forced Sleep</t>
         </is>
       </c>
       <c r="Q13" s="22" t="inlineStr">
         <is>
-          <t>Flip the room. The target is stunned next round.</t>
+          <t>Every enemy has to wait 2 more rounds for their special.</t>
         </is>
       </c>
       <c r="R13" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" s="22" t="n"/>
     </row>
     <row r="14" ht="26.85" customHeight="1" s="16">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Swamp Demon</t>
+          <t>Rui</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -1544,23 +1548,23 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Lesser demon</t>
+          <t>Lower Moon 5</t>
         </is>
       </c>
       <c r="E14" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J14" s="20" t="n">
         <v>1</v>
@@ -1583,23 +1587,23 @@
       </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>Swamp Dive</t>
+          <t>Cutting Thread Cage</t>
         </is>
       </c>
       <c r="Q14" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
+          <t>Strike for PWR and stun the target next round.</t>
         </is>
       </c>
       <c r="R14" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="22" t="n"/>
     </row>
     <row r="15" ht="26.85" customHeight="1" s="16">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Hand Demon</t>
+          <t>Kyogai</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
@@ -1614,20 +1618,20 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Final Selection</t>
+          <t>Former Lower Moon</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I15" s="20" t="n">
         <v>3</v>
@@ -1653,28 +1657,28 @@
       </c>
       <c r="P15" s="19" t="inlineStr">
         <is>
-          <t>Grasping Arms</t>
+          <t>Drum Room Spin</t>
         </is>
       </c>
       <c r="Q15" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Flip the room. The target is stunned next round.</t>
         </is>
       </c>
       <c r="R15" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S15" s="22" t="n"/>
     </row>
     <row r="16" ht="26.85" customHeight="1" s="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>Sekido (Anger)</t>
+          <t>Swamp Demon</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
@@ -1684,23 +1688,23 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Anger</t>
+          <t>Lesser demon</t>
         </is>
       </c>
       <c r="E16" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H16" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" s="20" t="n">
         <v>1</v>
@@ -1723,32 +1727,28 @@
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Lightning Staff</t>
+          <t>Swamp Dive</t>
         </is>
       </c>
       <c r="Q16" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4, ignores DEF.</t>
+          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
         </is>
       </c>
       <c r="R16" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S16" s="22" t="inlineStr">
-        <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="S16" s="22" t="n"/>
     </row>
     <row r="17" ht="26.85" customHeight="1" s="16">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Karaku (Joy)</t>
+          <t>Hand Demon</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
@@ -1758,20 +1758,20 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Joy</t>
+          <t>Final Selection</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I17" s="20" t="n">
         <v>3</v>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="P17" s="19" t="inlineStr">
         <is>
-          <t>Gale Fan</t>
+          <t>Grasping Arms</t>
         </is>
       </c>
       <c r="Q17" s="22" t="inlineStr">
@@ -1808,16 +1808,12 @@
       <c r="R17" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="S17" s="22" t="inlineStr">
-        <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
-        </is>
-      </c>
+      <c r="S17" s="22" t="n"/>
     </row>
     <row r="18" ht="26.85" customHeight="1" s="16">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Aizetsu (Sorrow)</t>
+          <t>Sekido (Anger)</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
@@ -1832,20 +1828,20 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Sorrow</t>
+          <t>Hantengu split · Anger</t>
         </is>
       </c>
       <c r="E18" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G18" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I18" s="20" t="n">
         <v>3</v>
@@ -1871,12 +1867,12 @@
       </c>
       <c r="P18" s="19" t="inlineStr">
         <is>
-          <t>Cross Spear</t>
+          <t>Lightning Staff</t>
         </is>
       </c>
       <c r="Q18" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4.</t>
+          <t>Every enemy takes 4, ignores DEF.</t>
         </is>
       </c>
       <c r="R18" s="20" t="n">
@@ -1884,14 +1880,14 @@
       </c>
       <c r="S18" s="22" t="inlineStr">
         <is>
-          <t>Appears when Sekido falls. Not drafted.</t>
+          <t>Appears when Hantengu falls. Not drafted.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="16">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Urogi (Pleasure)</t>
+          <t>Karaku (Joy)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -1906,23 +1902,23 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Pleasure</t>
+          <t>Hantengu split · Joy</t>
         </is>
       </c>
       <c r="E19" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H19" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="G19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="H19" s="20" t="n">
-        <v>11</v>
-      </c>
       <c r="I19" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="20" t="n">
         <v>1</v>
@@ -1945,12 +1941,12 @@
       </c>
       <c r="P19" s="19" t="inlineStr">
         <is>
-          <t>Sky Dive</t>
+          <t>Gale Fan</t>
         </is>
       </c>
       <c r="Q19" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Swoops down for PWR+2.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R19" s="20" t="n">
@@ -1958,48 +1954,48 @@
       </c>
       <c r="S19" s="22" t="inlineStr">
         <is>
-          <t>Appears when Karaku falls. Not drafted.</t>
+          <t>Appears when Hantengu falls. Not drafted.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26.85" customHeight="1" s="16">
-      <c r="A20" s="23" t="inlineStr">
-        <is>
-          <t>Gyomei Himejima (Mark)</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Aizetsu (Sorrow)</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Stone Hashira</t>
+          <t>Hantengu split · Sorrow</t>
         </is>
       </c>
       <c r="E20" s="20" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F20" s="20" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="H20" s="20" t="n">
         <v>9</v>
       </c>
       <c r="I20" s="20" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J20" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" s="21">
         <f>1/F20</f>
@@ -2019,61 +2015,61 @@
       </c>
       <c r="P20" s="19" t="inlineStr">
         <is>
-          <t>Volcanic Rock</t>
+          <t>Cross Spear</t>
         </is>
       </c>
       <c r="Q20" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Strike for PWR+4.</t>
         </is>
       </c>
       <c r="R20" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S20" s="22" t="inlineStr">
+        <is>
+          <t>Appears when Sekido falls. Not drafted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26.85" customHeight="1" s="16">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Urogi (Pleasure)</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Split form</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Hantengu split · Pleasure</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I21" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="S20" s="22" t="inlineStr">
-        <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="26.85" customHeight="1" s="16">
-      <c r="A21" s="23" t="inlineStr">
-        <is>
-          <t>Giyu Tomioka (Mark)</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>Slayer</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Water Hashira</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="F21" s="20" t="n">
-        <v>40</v>
-      </c>
-      <c r="G21" s="20" t="n">
-        <v>14</v>
-      </c>
-      <c r="H21" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I21" s="20" t="n">
-        <v>6</v>
-      </c>
       <c r="J21" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="21">
         <f>1/F21</f>
@@ -2093,27 +2089,27 @@
       </c>
       <c r="P21" s="19" t="inlineStr">
         <is>
-          <t>Dead Calm</t>
+          <t>Sky Dive</t>
         </is>
       </c>
       <c r="Q21" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Your whole team takes no damage this round.</t>
+          <t>Moves early. Swoops down for PWR+2.</t>
         </is>
       </c>
       <c r="R21" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S21" s="22" t="inlineStr">
         <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+          <t>Appears when Karaku falls. Not drafted.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26.85" customHeight="1" s="16">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>Muichiro Tokito (Mark)</t>
+          <t>Gyomei Himejima (Mark)</t>
         </is>
       </c>
       <c r="B22" s="23" t="inlineStr">
@@ -2128,23 +2124,23 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Mist Hashira</t>
+          <t>Stone Hashira</t>
         </is>
       </c>
       <c r="E22" s="20" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="I22" s="20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J22" s="20" t="n">
         <v>0</v>
@@ -2167,12 +2163,12 @@
       </c>
       <c r="P22" s="19" t="inlineStr">
         <is>
-          <t>Obscuring Clouds</t>
+          <t>Volcanic Rock</t>
         </is>
       </c>
       <c r="Q22" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R22" s="20" t="n">
@@ -2187,7 +2183,7 @@
     <row r="23" ht="15" customHeight="1" s="16">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>Sanemi Shinazugawa (Mark)</t>
+          <t>Giyu Tomioka (Mark)</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
@@ -2202,20 +2198,20 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Wind Hashira</t>
+          <t>Water Hashira</t>
         </is>
       </c>
       <c r="E23" s="20" t="n">
         <v>10</v>
       </c>
       <c r="F23" s="20" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G23" s="20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H23" s="20" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I23" s="20" t="n">
         <v>6</v>
@@ -2241,16 +2237,16 @@
       </c>
       <c r="P23" s="19" t="inlineStr">
         <is>
-          <t>Black Wind Mountain Mist</t>
+          <t>Dead Calm</t>
         </is>
       </c>
       <c r="Q23" s="22" t="inlineStr">
         <is>
-          <t>Strike your target and one other enemy for PWR.</t>
+          <t>Moves first. Your whole team takes no damage this round.</t>
         </is>
       </c>
       <c r="R23" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S23" s="22" t="inlineStr">
         <is>
@@ -2259,14 +2255,14 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="16">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>Giyu Tomioka</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Muichiro Tokito (Mark)</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
@@ -2276,20 +2272,20 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Water Hashira</t>
+          <t>Mist Hashira</t>
         </is>
       </c>
       <c r="E24" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F24" s="20" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G24" s="20" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H24" s="20" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I24" s="20" t="n">
         <v>5</v>
@@ -2315,28 +2311,32 @@
       </c>
       <c r="P24" s="19" t="inlineStr">
         <is>
-          <t>Dead Calm</t>
+          <t>Obscuring Clouds</t>
         </is>
       </c>
       <c r="Q24" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Your whole team takes no damage this round.</t>
+          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
         </is>
       </c>
       <c r="R24" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="S24" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S24" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="16">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Gyomei Himejima</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Sanemi Shinazugawa (Mark)</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
@@ -2346,23 +2346,23 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Stone Hashira</t>
+          <t>Wind Hashira</t>
         </is>
       </c>
       <c r="E25" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>42</v>
       </c>
       <c r="G25" s="20" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H25" s="20" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I25" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J25" s="20" t="n">
         <v>0</v>
@@ -2385,28 +2385,32 @@
       </c>
       <c r="P25" s="19" t="inlineStr">
         <is>
-          <t>Volcanic Rock</t>
+          <t>Black Wind Mountain Mist</t>
         </is>
       </c>
       <c r="Q25" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Strike your target and one other enemy for PWR.</t>
         </is>
       </c>
       <c r="R25" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S25" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S25" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="16">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>Mitsuri Kanroji (Mark)</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Giyu Tomioka</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
@@ -2416,20 +2420,20 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Love Hashira</t>
+          <t>Water Hashira</t>
         </is>
       </c>
       <c r="E26" s="20" t="n">
         <v>8</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I26" s="20" t="n">
         <v>5</v>
@@ -2455,32 +2459,28 @@
       </c>
       <c r="P26" s="19" t="inlineStr">
         <is>
-          <t>Catlove Shower</t>
+          <t>Dead Calm</t>
         </is>
       </c>
       <c r="Q26" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Moves first. Your whole team takes no damage this round.</t>
         </is>
       </c>
       <c r="R26" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S26" s="22" t="inlineStr">
-        <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="S26" s="22" t="n"/>
     </row>
     <row r="27" ht="26.85" customHeight="1" s="16">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>Obanai Iguro (Mark)</t>
-        </is>
-      </c>
-      <c r="B27" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Gyomei Himejima</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
@@ -2490,23 +2490,23 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Serpent Hashira</t>
+          <t>Stone Hashira</t>
         </is>
       </c>
       <c r="E27" s="20" t="n">
         <v>8</v>
       </c>
       <c r="F27" s="20" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G27" s="20" t="n">
         <v>13</v>
       </c>
       <c r="H27" s="20" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I27" s="20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J27" s="20" t="n">
         <v>0</v>
@@ -2529,27 +2529,23 @@
       </c>
       <c r="P27" s="19" t="inlineStr">
         <is>
-          <t>Twin-Headed Reptile</t>
+          <t>Volcanic Rock</t>
         </is>
       </c>
       <c r="Q27" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R27" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S27" s="22" t="inlineStr">
-        <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="S27" s="22" t="n"/>
     </row>
     <row r="28" ht="39.55" customHeight="1" s="16">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Tanjiro Kamado (Mark)</t>
+          <t>Mitsuri Kanroji (Mark)</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
@@ -2564,7 +2560,7 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Sun &amp; Water</t>
+          <t>Love Hashira</t>
         </is>
       </c>
       <c r="E28" s="20" t="n">
@@ -2574,10 +2570,10 @@
         <v>36</v>
       </c>
       <c r="G28" s="20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H28" s="20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I28" s="20" t="n">
         <v>5</v>
@@ -2603,12 +2599,12 @@
       </c>
       <c r="P28" s="19" t="inlineStr">
         <is>
-          <t>Hinokami Kagura</t>
+          <t>Catlove Shower</t>
         </is>
       </c>
       <c r="Q28" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+5, ignores DEF.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R28" s="20" t="n">
@@ -2621,14 +2617,14 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="16">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>Kyojuro Rengoku</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>Obanai Iguro (Mark)</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
@@ -2638,20 +2634,20 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Flame Hashira</t>
+          <t>Serpent Hashira</t>
         </is>
       </c>
       <c r="E29" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>34</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H29" s="20" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I29" s="20" t="n">
         <v>5</v>
@@ -2677,28 +2673,32 @@
       </c>
       <c r="P29" s="19" t="inlineStr">
         <is>
-          <t>Ninth Form: Rengoku</t>
+          <t>Twin-Headed Reptile</t>
         </is>
       </c>
       <c r="Q29" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+8.</t>
+          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
         </is>
       </c>
       <c r="R29" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S29" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S29" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="16">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>Muichiro Tokito</t>
-        </is>
-      </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>Tanjiro Kamado (Mark)</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
@@ -2708,23 +2708,23 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Mist Hashira</t>
+          <t>Sun &amp; Water</t>
         </is>
       </c>
       <c r="E30" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H30" s="20" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I30" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J30" s="20" t="n">
         <v>0</v>
@@ -2747,23 +2747,27 @@
       </c>
       <c r="P30" s="19" t="inlineStr">
         <is>
-          <t>Obscuring Clouds</t>
+          <t>Hinokami Kagura</t>
         </is>
       </c>
       <c r="Q30" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
+          <t>Strike for PWR+5, ignores DEF.</t>
         </is>
       </c>
       <c r="R30" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S30" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S30" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="16">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>Sanemi Shinazugawa</t>
+          <t>Kyojuro Rengoku</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
@@ -2778,11 +2782,11 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Wind Hashira</t>
+          <t>Flame Hashira</t>
         </is>
       </c>
       <c r="E31" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>34</v>
@@ -2791,7 +2795,7 @@
         <v>11</v>
       </c>
       <c r="H31" s="20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I31" s="20" t="n">
         <v>5</v>
@@ -2817,12 +2821,12 @@
       </c>
       <c r="P31" s="19" t="inlineStr">
         <is>
-          <t>Black Wind Mountain Mist</t>
+          <t>Ninth Form: Rengoku</t>
         </is>
       </c>
       <c r="Q31" s="22" t="inlineStr">
         <is>
-          <t>Strike your target and one other enemy for PWR.</t>
+          <t>Strike for PWR+8.</t>
         </is>
       </c>
       <c r="R31" s="20" t="n">
@@ -2833,7 +2837,7 @@
     <row r="32" ht="15" customHeight="1" s="16">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>Tengen Uzui</t>
+          <t>Muichiro Tokito</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
@@ -2848,23 +2852,23 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Sound Hashira</t>
+          <t>Mist Hashira</t>
         </is>
       </c>
       <c r="E32" s="20" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G32" s="20" t="n">
         <v>10</v>
       </c>
       <c r="H32" s="20" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I32" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J32" s="20" t="n">
         <v>0</v>
@@ -2887,12 +2891,12 @@
       </c>
       <c r="P32" s="19" t="inlineStr">
         <is>
-          <t>Constant Resounding Slashes</t>
+          <t>Obscuring Clouds</t>
         </is>
       </c>
       <c r="Q32" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−2.</t>
+          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
         </is>
       </c>
       <c r="R32" s="20" t="n">
@@ -2903,7 +2907,7 @@
     <row r="33" ht="26.85" customHeight="1" s="16">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>Mitsuri Kanroji</t>
+          <t>Sanemi Shinazugawa</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -2918,23 +2922,23 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Love Hashira</t>
+          <t>Wind Hashira</t>
         </is>
       </c>
       <c r="E33" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H33" s="20" t="n">
         <v>9</v>
       </c>
       <c r="I33" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J33" s="20" t="n">
         <v>0</v>
@@ -2957,12 +2961,12 @@
       </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
-          <t>Catlove Shower</t>
+          <t>Black Wind Mountain Mist</t>
         </is>
       </c>
       <c r="Q33" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Strike your target and one other enemy for PWR.</t>
         </is>
       </c>
       <c r="R33" s="20" t="n">
@@ -2973,7 +2977,7 @@
     <row r="34" ht="15" customHeight="1" s="16">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>Obanai Iguro</t>
+          <t>Tengen Uzui</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -2988,23 +2992,23 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Serpent Hashira</t>
+          <t>Sound Hashira</t>
         </is>
       </c>
       <c r="E34" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="G34" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H34" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I34" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F34" s="20" t="n">
-        <v>26</v>
-      </c>
-      <c r="G34" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="H34" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I34" s="20" t="n">
-        <v>4</v>
       </c>
       <c r="J34" s="20" t="n">
         <v>0</v>
@@ -3027,12 +3031,12 @@
       </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
-          <t>Twin-Headed Reptile</t>
+          <t>Constant Resounding Slashes</t>
         </is>
       </c>
       <c r="Q34" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
+          <t>Every enemy takes PWR−2.</t>
         </is>
       </c>
       <c r="R34" s="20" t="n">
@@ -3043,7 +3047,7 @@
     <row r="35" ht="26.85" customHeight="1" s="16">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>Shinobu Kocho</t>
+          <t>Mitsuri Kanroji</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -3058,23 +3062,23 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Insect Hashira</t>
+          <t>Love Hashira</t>
         </is>
       </c>
       <c r="E35" s="20" t="n">
         <v>5</v>
       </c>
       <c r="F35" s="20" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G35" s="20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H35" s="20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I35" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J35" s="20" t="n">
         <v>0</v>
@@ -3097,27 +3101,23 @@
       </c>
       <c r="P35" s="19" t="inlineStr">
         <is>
-          <t>Wisteria Poison</t>
+          <t>Catlove Shower</t>
         </is>
       </c>
       <c r="Q35" s="22" t="inlineStr">
         <is>
-          <t>Poison a target for 3 rounds: 6/round to demons, 3/round to humans.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R35" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S35" s="22" t="inlineStr">
-        <is>
-          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match.</t>
-        </is>
-      </c>
+      <c r="S35" s="22" t="n"/>
     </row>
     <row r="36" ht="26.85" customHeight="1" s="16">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>Tanjiro Kamado</t>
+          <t>Obanai Iguro</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -3132,20 +3132,20 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Sun &amp; Water</t>
+          <t>Serpent Hashira</t>
         </is>
       </c>
       <c r="E36" s="20" t="n">
         <v>5</v>
       </c>
       <c r="F36" s="20" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G36" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H36" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I36" s="20" t="n">
         <v>4</v>
@@ -3171,12 +3171,12 @@
       </c>
       <c r="P36" s="19" t="inlineStr">
         <is>
-          <t>Hinokami Kagura</t>
+          <t>Twin-Headed Reptile</t>
         </is>
       </c>
       <c r="Q36" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+5, ignores DEF.</t>
+          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
         </is>
       </c>
       <c r="R36" s="20" t="n">
@@ -3187,7 +3187,7 @@
     <row r="37" ht="26.85" customHeight="1" s="16">
       <c r="A37" s="19" t="inlineStr">
         <is>
-          <t>Inosuke Hashibira</t>
+          <t>Shinobu Kocho</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -3202,20 +3202,20 @@
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Beast</t>
+          <t>Insect Hashira</t>
         </is>
       </c>
       <c r="E37" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G37" s="20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H37" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I37" s="20" t="n">
         <v>3</v>
@@ -3241,23 +3241,27 @@
       </c>
       <c r="P37" s="19" t="inlineStr">
         <is>
-          <t>Fang Frenzy</t>
+          <t>Wisteria Poison</t>
         </is>
       </c>
       <c r="Q37" s="22" t="inlineStr">
         <is>
-          <t>Two wild strikes of PWR−1 at random enemies.</t>
+          <t>Poison a target for 3 rounds: 6/round to demons, 3/round to humans.</t>
         </is>
       </c>
       <c r="R37" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S37" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S37" s="22" t="inlineStr">
+        <is>
+          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>Kanao Tsuyuri</t>
+          <t>Tanjiro Kamado</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -3272,23 +3276,23 @@
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Flower</t>
+          <t>Sun &amp; Water</t>
         </is>
       </c>
       <c r="E38" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G38" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H38" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I38" s="20" t="n">
         <v>4</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="G38" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="H38" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J38" s="20" t="n">
         <v>0</v>
@@ -3311,12 +3315,12 @@
       </c>
       <c r="P38" s="19" t="inlineStr">
         <is>
-          <t>Equinoctial Vermilion Eye</t>
+          <t>Hinokami Kagura</t>
         </is>
       </c>
       <c r="Q38" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Strike for PWR+4.</t>
+          <t>Strike for PWR+5, ignores DEF.</t>
         </is>
       </c>
       <c r="R38" s="20" t="n">
@@ -3327,7 +3331,7 @@
     <row r="39" ht="15" customHeight="1" s="16">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>Nezuko Kamado</t>
+          <t>Inosuke Hashibira</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -3337,31 +3341,31 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Beast</t>
         </is>
       </c>
       <c r="E39" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F39" s="20" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H39" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I39" s="20" t="n">
         <v>3</v>
       </c>
       <c r="J39" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" s="21">
         <f>1/F39</f>
@@ -3381,23 +3385,23 @@
       </c>
       <c r="P39" s="19" t="inlineStr">
         <is>
-          <t>Exploding Blood</t>
+          <t>Fang Frenzy</t>
         </is>
       </c>
       <c r="Q39" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 5, ignores DEF.</t>
+          <t>Two wild strikes of PWR−1 at random enemies.</t>
         </is>
       </c>
       <c r="R39" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S39" s="22" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="16">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>Sakonji Urokodaki</t>
+          <t>Kanao Tsuyuri</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -3412,23 +3416,23 @@
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Former Water Hashira</t>
+          <t>Flower</t>
         </is>
       </c>
       <c r="E40" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G40" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H40" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I40" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J40" s="20" t="n">
         <v>0</v>
@@ -3451,61 +3455,57 @@
       </c>
       <c r="P40" s="19" t="inlineStr">
         <is>
-          <t>Water Wheel</t>
+          <t>Equinoctial Vermilion Eye</t>
         </is>
       </c>
       <c r="Q40" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Moves early. Strike for PWR+4.</t>
         </is>
       </c>
       <c r="R40" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S40" s="22" t="inlineStr">
-        <is>
-          <t>Mentor: Tanjiro and Giyu on his team get +1 DEF.</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="S40" s="22" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="16">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>Tengen Uzui (Retired)</t>
+          <t>Nezuko Kamado</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Retired</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Former Sound Hashira</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="E41" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H41" s="20" t="n">
         <v>7</v>
       </c>
       <c r="I41" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J41" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" s="21">
         <f>1/F41</f>
@@ -3525,27 +3525,23 @@
       </c>
       <c r="P41" s="19" t="inlineStr">
         <is>
-          <t>Bodyguard</t>
+          <t>Exploding Blood</t>
         </is>
       </c>
       <c r="Q41" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Shields an ally (or himself): they count as Defending this round and take half damage.</t>
+          <t>Every enemy takes 5, ignores DEF.</t>
         </is>
       </c>
       <c r="R41" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S41" s="22" t="inlineStr">
-        <is>
-          <t>Retired: lost a hand and an eye, so he no longer counts as a Hashira.</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="S41" s="22" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="16">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>Zenitsu Agatsuma</t>
+          <t>Sabito &amp; Makomo</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -3560,14 +3556,14 @@
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>Thunder</t>
+          <t>Spirits · Urokodaki's students</t>
         </is>
       </c>
       <c r="E42" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F42" s="20" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G42" s="20" t="n">
         <v>7</v>
@@ -3576,7 +3572,7 @@
         <v>10</v>
       </c>
       <c r="I42" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J42" s="20" t="n">
         <v>0</v>
@@ -3599,23 +3595,27 @@
       </c>
       <c r="P42" s="19" t="inlineStr">
         <is>
-          <t>Thunderclap and Flash</t>
+          <t>Spirit Training</t>
         </is>
       </c>
       <c r="Q42" s="22" t="inlineStr">
         <is>
-          <t>Always moves first. Strike for PWR×2.</t>
+          <t>Train an ally (or themselves): +2 PWR for the rest of the match.</t>
         </is>
       </c>
       <c r="R42" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S42" s="22" t="n"/>
+      <c r="S42" s="22" t="inlineStr">
+        <is>
+          <t>Urokodaki's students: they get his Mentor bonus too.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>Genya Shinazugawa</t>
+          <t>Sakonji Urokodaki</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -3630,23 +3630,23 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Demon eater</t>
+          <t>Former Water Hashira</t>
         </is>
       </c>
       <c r="E43" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F43" s="20" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G43" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H43" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I43" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J43" s="20" t="n">
         <v>0</v>
@@ -3669,57 +3669,61 @@
       </c>
       <c r="P43" s="19" t="inlineStr">
         <is>
-          <t>Demon Consumption</t>
+          <t>Water Wheel</t>
         </is>
       </c>
       <c r="Q43" s="22" t="inlineStr">
         <is>
-          <t>Heal 8 and gain +2 PWR for the rest of the match.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R43" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S43" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S43" s="22" t="inlineStr">
+        <is>
+          <t>Mentor: Tanjiro, Giyu and Sabito &amp; Makomo on his team get +1 DEF.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>Tamayo</t>
+          <t>Tengen Uzui (Retired)</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>Physician · Demon ally</t>
+          <t>Former Sound Hashira</t>
         </is>
       </c>
       <c r="E44" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H44" s="20" t="n">
         <v>7</v>
       </c>
       <c r="I44" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J44" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" s="21">
         <f>1/F44</f>
@@ -3739,12 +3743,12 @@
       </c>
       <c r="P44" s="19" t="inlineStr">
         <is>
-          <t>Healing Blood Art</t>
+          <t>Bodyguard</t>
         </is>
       </c>
       <c r="Q44" s="22" t="inlineStr">
         <is>
-          <t>Heal an ally (or herself) for 10 and cure poison.</t>
+          <t>Moves first. Shields an ally (or himself): they count as Defending this round and take half damage.</t>
         </is>
       </c>
       <c r="R44" s="20" t="n">
@@ -3752,14 +3756,14 @@
       </c>
       <c r="S44" s="22" t="inlineStr">
         <is>
-          <t>Anti-Muzan Medicine: an enemy Muzan's regeneration drops by 2.</t>
+          <t>Retired: lost a hand and an eye, so he no longer counts as a Hashira.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>Yushiro</t>
+          <t>Zenitsu Agatsuma</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -3769,31 +3773,31 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Tamayo's guardian · Demon ally</t>
+          <t>Thunder</t>
         </is>
       </c>
       <c r="E45" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F45" s="20" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H45" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I45" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J45" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" s="21">
         <f>1/F45</f>
@@ -3813,12 +3817,12 @@
       </c>
       <c r="P45" s="19" t="inlineStr">
         <is>
-          <t>Concealment Talisman</t>
+          <t>Thunderclap and Flash</t>
         </is>
       </c>
       <c r="Q45" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Hide an ally (or himself): attacks against them miss this round.</t>
+          <t>Always moves first. Strike for PWR×2.</t>
         </is>
       </c>
       <c r="R45" s="20" t="n">
@@ -3829,7 +3833,7 @@
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Kagaya Ubuyashiki</t>
+          <t>Genya Shinazugawa</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -3844,23 +3848,23 @@
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>Corps Master</t>
+          <t>Demon eater</t>
         </is>
       </c>
       <c r="E46" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" s="20" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H46" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I46" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J46" s="20" t="n">
         <v>0</v>
@@ -3883,27 +3887,23 @@
       </c>
       <c r="P46" s="19" t="inlineStr">
         <is>
-          <t>Words of Resolve</t>
+          <t>Demon Consumption</t>
         </is>
       </c>
       <c r="Q46" s="22" t="inlineStr">
         <is>
-          <t>Every ally, himself included, heals 4.</t>
+          <t>Heal 8 and gain +2 PWR for the rest of the match.</t>
         </is>
       </c>
       <c r="R46" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S46" s="22" t="inlineStr">
-        <is>
-          <t>Master of the Corps: every Hashira on his team gets +1 DEF.</t>
-        </is>
-      </c>
+      <c r="S46" s="22" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Tamayo</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -3913,31 +3913,31 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Water · rank and file</t>
+          <t>Physician · Demon ally</t>
         </is>
       </c>
       <c r="E47" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I47" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="20" t="n">
         <v>2</v>
-      </c>
-      <c r="F47" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="G47" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H47" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="I47" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J47" s="20" t="n">
-        <v>0</v>
       </c>
       <c r="K47" s="21">
         <f>1/F47</f>
@@ -3957,12 +3957,12 @@
       </c>
       <c r="P47" s="19" t="inlineStr">
         <is>
-          <t>Water Surface Slash</t>
+          <t>Healing Blood Art</t>
         </is>
       </c>
       <c r="Q47" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+2.</t>
+          <t>Heal an ally (or herself) for 10 and cure poison.</t>
         </is>
       </c>
       <c r="R47" s="20" t="n">
@@ -3970,49 +3970,267 @@
       </c>
       <c r="S47" s="22" t="inlineStr">
         <is>
+          <t>Anti-Muzan Medicine: an enemy Muzan's regeneration drops by 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>Yushiro</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>Demon ally</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>Tamayo's guardian · Demon ally</t>
+        </is>
+      </c>
+      <c r="E48" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I48" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" s="21">
+        <f>1/F48</f>
+        <v/>
+      </c>
+      <c r="L48" s="21">
+        <f>J48/F48</f>
+        <v/>
+      </c>
+      <c r="M48" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="20" t="n"/>
+      <c r="O48" s="21">
+        <f>IF(N48="","",N48/F48)</f>
+        <v/>
+      </c>
+      <c r="P48" s="19" t="inlineStr">
+        <is>
+          <t>Concealment Talisman</t>
+        </is>
+      </c>
+      <c r="Q48" s="22" t="inlineStr">
+        <is>
+          <t>Moves first. Hide an ally (or himself): attacks against them miss this round.</t>
+        </is>
+      </c>
+      <c r="R48" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S48" s="22" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>Kagaya Ubuyashiki</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Corps Master</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="21">
+        <f>1/F49</f>
+        <v/>
+      </c>
+      <c r="L49" s="21">
+        <f>J49/F49</f>
+        <v/>
+      </c>
+      <c r="M49" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N49" s="20" t="n"/>
+      <c r="O49" s="21">
+        <f>IF(N49="","",N49/F49)</f>
+        <v/>
+      </c>
+      <c r="P49" s="19" t="inlineStr">
+        <is>
+          <t>Words of Resolve</t>
+        </is>
+      </c>
+      <c r="Q49" s="22" t="inlineStr">
+        <is>
+          <t>Every ally, himself included, heals 4.</t>
+        </is>
+      </c>
+      <c r="R49" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S49" s="22" t="inlineStr">
+        <is>
+          <t>Master of the Corps: every Hashira on his team gets +1 DEF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>Murata</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>Water · rank and file</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G50" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H50" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="I50" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="21">
+        <f>1/F50</f>
+        <v/>
+      </c>
+      <c r="L50" s="21">
+        <f>J50/F50</f>
+        <v/>
+      </c>
+      <c r="M50" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" s="20" t="n"/>
+      <c r="O50" s="21">
+        <f>IF(N50="","",N50/F50)</f>
+        <v/>
+      </c>
+      <c r="P50" s="19" t="inlineStr">
+        <is>
+          <t>Water Surface Slash</t>
+        </is>
+      </c>
+      <c r="Q50" s="22" t="inlineStr">
+        <is>
+          <t>Strike for PWR+2.</t>
+        </is>
+      </c>
+      <c r="R50" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="S50" s="22" t="inlineStr">
+        <is>
           <t>Somehow Survives: the first hit that would knock him out leaves him at 1 HP instead.</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="A49" s="24" t="inlineStr">
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="25" t="inlineStr">
-        <is>
-          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 24 2026). Black cells are formulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="25" t="inlineStr">
-        <is>
-          <t>"1 HP = % of bar": how much of a fighter's bar one point of damage removes. Smaller = tankier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="25" t="inlineStr">
-        <is>
-          <t>Pink rows are Mark-awakened versions (+8 HP, +4 PWR, +2 SPD, +1 DEF, special 1 round faster; cost set per character). Gold rows are Legends.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Retired Tengen is the other version of Tengen (one or the other is dealt).</t>
+          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 24 2026). Black cells are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t>"1 HP = % of bar": how much of a fighter's bar one point of damage removes. Smaller = tankier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>Pink rows are Mark-awakened versions (+8 HP, +4 PWR, +2 SPD, +1 DEF, special 1 round faster; cost set per character). Gold rows are Legends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Retired Tengen and Final-Form Muzan are second versions (one or the other is dealt).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S47"/>
-  <conditionalFormatting sqref="F2:F47">
+  <autoFilter ref="A1:S50"/>
+  <conditionalFormatting sqref="F2:F50">
     <cfRule type="dataBar" priority="1">
       <dataBar minLength="10" maxLength="90" showValue="1">
         <cfvo type="num" val="0"/>
@@ -4094,7 +4312,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="29">
-        <f>IF(A5="","",INDEX(Roster!$F$2:$F$47,MATCH(A5,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A5="","",INDEX(Roster!$F$2:$F$50,MATCH(A5,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D5" s="30">
@@ -4116,7 +4334,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="29">
-        <f>IF(A6="","",INDEX(Roster!$F$2:$F$47,MATCH(A6,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A6="","",INDEX(Roster!$F$2:$F$50,MATCH(A6,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D6" s="30">
@@ -4138,7 +4356,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="29">
-        <f>IF(A7="","",INDEX(Roster!$F$2:$F$47,MATCH(A7,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A7="","",INDEX(Roster!$F$2:$F$50,MATCH(A7,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D7" s="30">
@@ -4160,7 +4378,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="29">
-        <f>IF(A8="","",INDEX(Roster!$F$2:$F$47,MATCH(A8,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A8="","",INDEX(Roster!$F$2:$F$50,MATCH(A8,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D8" s="30">
@@ -4182,7 +4400,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="29">
-        <f>IF(A9="","",INDEX(Roster!$F$2:$F$47,MATCH(A9,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A9="","",INDEX(Roster!$F$2:$F$50,MATCH(A9,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D9" s="30">
@@ -4198,7 +4416,7 @@
       <c r="A10" s="28" t="n"/>
       <c r="B10" s="28" t="n"/>
       <c r="C10" s="29">
-        <f>IF(A10="","",INDEX(Roster!$F$2:$F$47,MATCH(A10,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A10="","",INDEX(Roster!$F$2:$F$50,MATCH(A10,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D10" s="30">
@@ -4214,7 +4432,7 @@
       <c r="A11" s="28" t="n"/>
       <c r="B11" s="28" t="n"/>
       <c r="C11" s="29">
-        <f>IF(A11="","",INDEX(Roster!$F$2:$F$47,MATCH(A11,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A11="","",INDEX(Roster!$F$2:$F$50,MATCH(A11,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D11" s="30">
@@ -4230,7 +4448,7 @@
       <c r="A12" s="28" t="n"/>
       <c r="B12" s="28" t="n"/>
       <c r="C12" s="29">
-        <f>IF(A12="","",INDEX(Roster!$F$2:$F$47,MATCH(A12,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A12="","",INDEX(Roster!$F$2:$F$50,MATCH(A12,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D12" s="30">
@@ -4246,7 +4464,7 @@
       <c r="A13" s="28" t="n"/>
       <c r="B13" s="28" t="n"/>
       <c r="C13" s="29">
-        <f>IF(A13="","",INDEX(Roster!$F$2:$F$47,MATCH(A13,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A13="","",INDEX(Roster!$F$2:$F$50,MATCH(A13,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D13" s="30">
@@ -4262,7 +4480,7 @@
       <c r="A14" s="28" t="n"/>
       <c r="B14" s="28" t="n"/>
       <c r="C14" s="29">
-        <f>IF(A14="","",INDEX(Roster!$F$2:$F$47,MATCH(A14,Roster!$A$2:$A$47,0)))</f>
+        <f>IF(A14="","",INDEX(Roster!$F$2:$F$50,MATCH(A14,Roster!$A$2:$A$50,0)))</f>
         <v/>
       </c>
       <c r="D14" s="30">
@@ -4297,7 +4515,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="A5:A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>Roster!$A$2:$A$47</formula1>
+      <formula1>Roster!$A$2:$A$50</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
30-point drafts deal 14 stronger characters; Muzan's whips ignore DEF
30-point pools favour pricier characters and Mark versions while Yoriichi and
Final-Form Muzan keep hard-pull odds. Muzan's and Final Muzan's whips now
ignore DEF at lower base damage, which keeps them strong against the high-DEF
teams 30-point games produce.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -880,7 +880,7 @@
       </c>
       <c r="Q4" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3, and he heals 3 for each enemy hit.</t>
+          <t>Every enemy takes PWR−6, ignores DEF, and he heals 3 for each enemy hit.</t>
         </is>
       </c>
       <c r="R4" s="20" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="Q5" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−4, and Muzan heals 2 for each enemy hit.</t>
+          <t>Every enemy takes PWR−7, ignores DEF, and Muzan heals 2 for each enemy hit.</t>
         </is>
       </c>
       <c r="R5" s="20" t="n">
@@ -4274,7 +4274,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -4492,7 +4491,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Buff Doma so Upper Moon 2 outranks Akaza
11 pts, 44 HP, 14 PWR, 11 SPD, 6 DEF, regen 3; Frozen Lotus now deals PWR−4
to every enemy, ignoring DEF, instead of a flat 8.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -1198,22 +1198,22 @@
         </is>
       </c>
       <c r="E9" s="20" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G9" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="H9" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="H9" s="20" t="n">
-        <v>9</v>
-      </c>
       <c r="I9" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="21">
         <f>1/F9</f>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="Q9" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 8, ignores DEF.</t>
+          <t>Every enemy takes PWR−4, ignores DEF.</t>
         </is>
       </c>
       <c r="R9" s="20" t="n">

</xml_diff>

<commit_message>
Back-pocket helpers and budget-aware pool notes
Chachamaru, Kasugai Crow and Muscle Mice: 1 pt helpers offered every draft that
don't take a fighter slot and are used once on a chosen round. Chachamaru
heals the team by half their current health, the Crow reveals the enemy's
moves and lets you change yours, the Mice give the team +2 PWR for the round.
Pool notes now hide pairings no team could afford in the match's points.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -11,7 +11,7 @@
     <sheet name="HP % Calculator" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S56"/>
+  <dimension ref="A1:S59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="15" min="1" max="1"/>
@@ -1035,7 +1035,7 @@
     <row r="7" ht="15" customHeight="1" s="16">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Akaza</t>
+          <t>Doma</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
@@ -1050,26 +1050,26 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 3</t>
+          <t>Upper Moon 2</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="21">
         <f>1/F7</f>
@@ -1089,12 +1089,12 @@
       </c>
       <c r="P7" s="19" t="inlineStr">
         <is>
-          <t>Destructive Death</t>
+          <t>Frozen Lotus</t>
         </is>
       </c>
       <c r="Q7" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+6.</t>
+          <t>Every enemy takes PWR−4, ignores DEF.</t>
         </is>
       </c>
       <c r="R7" s="20" t="n">
@@ -1105,7 +1105,7 @@
     <row r="8" ht="26.85" customHeight="1" s="16">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>Hantengu</t>
+          <t>Akaza</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
@@ -1120,26 +1120,26 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 4</t>
+          <t>Upper Moon 3</t>
         </is>
       </c>
       <c r="E8" s="20" t="n">
         <v>9</v>
       </c>
       <c r="F8" s="20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="21">
         <f>1/F8</f>
@@ -1159,27 +1159,23 @@
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Cowering Hide</t>
+          <t>Destructive Death</t>
         </is>
       </c>
       <c r="Q8" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
+          <t>Strike for PWR+6.</t>
         </is>
       </c>
       <c r="R8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S8" s="22" t="inlineStr">
-        <is>
-          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
-        </is>
-      </c>
+      <c r="S8" s="22" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="16">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Doma</t>
+          <t>Hantengu</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -1194,26 +1190,26 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 2</t>
+          <t>Upper Moon 4</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" s="21">
         <f>1/F9</f>
@@ -1233,18 +1229,22 @@
       </c>
       <c r="P9" s="19" t="inlineStr">
         <is>
-          <t>Frozen Lotus</t>
+          <t>Cowering Hide</t>
         </is>
       </c>
       <c r="Q9" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−4, ignores DEF.</t>
+          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
         </is>
       </c>
       <c r="R9" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S9" s="22" t="n"/>
+      <c r="S9" s="22" t="inlineStr">
+        <is>
+          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="16">
       <c r="A10" s="19" t="inlineStr">
@@ -4192,45 +4192,198 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>Chachamaru</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Tamayo's cat · back-pocket helper</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="20" t="n"/>
+      <c r="G51" s="20" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="20" t="n"/>
+      <c r="K51" s="21" t="n"/>
+      <c r="L51" s="21" t="n"/>
+      <c r="M51" s="20" t="n"/>
+      <c r="N51" s="20" t="n"/>
+      <c r="O51" s="21" t="n"/>
+      <c r="P51" s="19" t="inlineStr">
+        <is>
+          <t>Medicine Delivery</t>
+        </is>
+      </c>
+      <c r="Q51" s="22" t="inlineStr">
+        <is>
+          <t>Every fighter on your team heals half of their current health (50% becomes 75%).</t>
+        </is>
+      </c>
+      <c r="R51" s="20" t="n"/>
+      <c r="S51" s="22" t="inlineStr">
+        <is>
+          <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
-      <c r="A52" s="24" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>Kasugai Crow</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>Messenger crow · back-pocket helper</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="20" t="n"/>
+      <c r="G52" s="20" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="20" t="n"/>
+      <c r="K52" s="21" t="n"/>
+      <c r="L52" s="21" t="n"/>
+      <c r="M52" s="20" t="n"/>
+      <c r="N52" s="20" t="n"/>
+      <c r="O52" s="21" t="n"/>
+      <c r="P52" s="19" t="inlineStr">
+        <is>
+          <t>Scouting Report</t>
+        </is>
+      </c>
+      <c r="Q52" s="22" t="inlineStr">
+        <is>
+          <t>After both sides lock in, the crow shows you the enemy's moves, and you can change yours before the round plays.</t>
+        </is>
+      </c>
+      <c r="R52" s="20" t="n"/>
+      <c r="S52" s="22" t="inlineStr">
+        <is>
+          <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>Muscle Mice</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>Tengen's mice · back-pocket helper</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="20" t="n"/>
+      <c r="G53" s="20" t="n"/>
+      <c r="H53" s="20" t="n"/>
+      <c r="I53" s="20" t="n"/>
+      <c r="J53" s="20" t="n"/>
+      <c r="K53" s="21" t="n"/>
+      <c r="L53" s="21" t="n"/>
+      <c r="M53" s="20" t="n"/>
+      <c r="N53" s="20" t="n"/>
+      <c r="O53" s="21" t="n"/>
+      <c r="P53" s="19" t="inlineStr">
+        <is>
+          <t>Flex!</t>
+        </is>
+      </c>
+      <c r="Q53" s="22" t="inlineStr">
+        <is>
+          <t>Every fighter on your team gets +2 PWR for this round.</t>
+        </is>
+      </c>
+      <c r="R53" s="20" t="n"/>
+      <c r="S53" s="22" t="inlineStr">
+        <is>
+          <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55">
+      <c r="A55" s="24" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="25" t="inlineStr">
-        <is>
-          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 24 2026). Black cells are formulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>"1 HP = % of bar": how much of a fighter's bar one point of damage removes. Smaller = tankier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>Pink rows are Mark-awakened versions (+8 HP, +4 PWR, +2 SPD, +1 DEF, special 1 round faster; cost set per character). Gold rows are Legends.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Retired Tengen and Final-Form Muzan are second versions (one or the other is dealt).</t>
+          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 25 2026). Black cells are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>"1 HP = % of bar": how much of a fighter's bar one point of damage removes. Smaller = tankier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>Pink rows are Mark-awakened versions (+8 HP, +4 PWR, +2 SPD, +1 DEF, special 1 round faster; cost set per character). Gold rows are Legends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Retired Tengen and Final-Form Muzan are second versions (one or the other is dealt). Helpers (1 pt) sit in the back pocket and have no fighting stats.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S50"/>
-  <conditionalFormatting sqref="F2:F50">
+  <autoFilter ref="A1:S53"/>
+  <conditionalFormatting sqref="F2:F53">
     <cfRule type="dataBar" priority="1">
       <dataBar minLength="10" maxLength="90" showValue="1">
         <cfvo type="num" val="0"/>
@@ -4274,6 +4427,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -4311,7 +4465,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="29">
-        <f>IF(A5="","",INDEX(Roster!$F$2:$F$50,MATCH(A5,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A5="","",INDEX(Roster!$F$2:$F$53,MATCH(A5,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D5" s="30">
@@ -4333,7 +4487,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="29">
-        <f>IF(A6="","",INDEX(Roster!$F$2:$F$50,MATCH(A6,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A6="","",INDEX(Roster!$F$2:$F$53,MATCH(A6,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D6" s="30">
@@ -4355,7 +4509,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="29">
-        <f>IF(A7="","",INDEX(Roster!$F$2:$F$50,MATCH(A7,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A7="","",INDEX(Roster!$F$2:$F$53,MATCH(A7,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D7" s="30">
@@ -4377,7 +4531,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="29">
-        <f>IF(A8="","",INDEX(Roster!$F$2:$F$50,MATCH(A8,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A8="","",INDEX(Roster!$F$2:$F$53,MATCH(A8,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D8" s="30">
@@ -4399,7 +4553,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="29">
-        <f>IF(A9="","",INDEX(Roster!$F$2:$F$50,MATCH(A9,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A9="","",INDEX(Roster!$F$2:$F$53,MATCH(A9,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D9" s="30">
@@ -4415,7 +4569,7 @@
       <c r="A10" s="28" t="n"/>
       <c r="B10" s="28" t="n"/>
       <c r="C10" s="29">
-        <f>IF(A10="","",INDEX(Roster!$F$2:$F$50,MATCH(A10,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A10="","",INDEX(Roster!$F$2:$F$53,MATCH(A10,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D10" s="30">
@@ -4431,7 +4585,7 @@
       <c r="A11" s="28" t="n"/>
       <c r="B11" s="28" t="n"/>
       <c r="C11" s="29">
-        <f>IF(A11="","",INDEX(Roster!$F$2:$F$50,MATCH(A11,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A11="","",INDEX(Roster!$F$2:$F$53,MATCH(A11,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D11" s="30">
@@ -4447,7 +4601,7 @@
       <c r="A12" s="28" t="n"/>
       <c r="B12" s="28" t="n"/>
       <c r="C12" s="29">
-        <f>IF(A12="","",INDEX(Roster!$F$2:$F$50,MATCH(A12,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A12="","",INDEX(Roster!$F$2:$F$53,MATCH(A12,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D12" s="30">
@@ -4463,7 +4617,7 @@
       <c r="A13" s="28" t="n"/>
       <c r="B13" s="28" t="n"/>
       <c r="C13" s="29">
-        <f>IF(A13="","",INDEX(Roster!$F$2:$F$50,MATCH(A13,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A13="","",INDEX(Roster!$F$2:$F$53,MATCH(A13,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D13" s="30">
@@ -4479,7 +4633,7 @@
       <c r="A14" s="28" t="n"/>
       <c r="B14" s="28" t="n"/>
       <c r="C14" s="29">
-        <f>IF(A14="","",INDEX(Roster!$F$2:$F$50,MATCH(A14,Roster!$A$2:$A$50,0)))</f>
+        <f>IF(A14="","",INDEX(Roster!$F$2:$F$53,MATCH(A14,Roster!$A$2:$A$53,0)))</f>
         <v/>
       </c>
       <c r="D14" s="30">
@@ -4491,6 +4645,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
@@ -4513,7 +4668,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="A5:A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>Roster!$A$2:$A$50</formula1>
+      <formula1>Roster!$A$2:$A$53</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Akaza doesn't devour Shinobu
Shinobu's Wisteria Body poisons the demon that knocks her out, except Akaza,
who never eats women. Card text and pool note updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -3254,7 +3254,7 @@
       </c>
       <c r="S37" s="22" t="inlineStr">
         <is>
-          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match.</t>
+          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match. (Not Akaza: he never eats women.)</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -4645,7 +4644,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Balance: fix Gyomei, Rengoku, Akaza, Hand Demon; Genya to 4 pts
Gyomei's Volcanic Rock now deals fixed damage that ignores DEF (9, Mark 11) and he gets +1 SPD.
Rengoku +4 HP +2 SPD, Akaza +4 HP, Hand Demon -2 HP -1 PWR, Genya 4 pts with 30 HP / 7 SPD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -1127,7 +1127,7 @@
         <v>9</v>
       </c>
       <c r="F8" s="20" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G8" s="20" t="n">
         <v>13</v>
@@ -1765,10 +1765,10 @@
         <v>2</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H17" s="20" t="n">
         <v>4</v>
@@ -2137,7 +2137,7 @@
         <v>17</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>8</v>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="Q22" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Every enemy takes 11, ignores DEF.</t>
         </is>
       </c>
       <c r="R22" s="20" t="n">
@@ -2503,7 +2503,7 @@
         <v>13</v>
       </c>
       <c r="H27" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I27" s="20" t="n">
         <v>7</v>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="Q27" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Every enemy takes 9, ignores DEF.</t>
         </is>
       </c>
       <c r="R27" s="20" t="n">
@@ -2789,13 +2789,13 @@
         <v>7</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G31" s="20" t="n">
         <v>11</v>
       </c>
       <c r="H31" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I31" s="20" t="n">
         <v>5</v>
@@ -3852,16 +3852,16 @@
         </is>
       </c>
       <c r="E46" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46" s="20" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G46" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H46" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I46" s="20" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Add Nakime, Susamaru, Yahaba, Kanae, Demon King Tanjiro, Awakened Nezuko, Zohakuten, Yoriichi Type Zero, Hotaru; split Gyutaro and Daki
- Nakime has no Attack: Biwa Strum (enemy acts last) and Castle Shift (enemy away for the round); flees if left alone
- Gyutaro and Daki are separate cards; Two as One: Gyutaro +2 PWR and each can get back up once while the other stands
- Susamaru + Yahaba (Temari & Arrows), Kanae (Kocho Sisters, Kanao's teacher), Type Zero (triple strike, Muichiro partner)
- Demon King Tanjiro (rare, sun-proof), Awakened Nezuko (can't Defend), Zohakuten (Hantengu's other version)
- Hotaru helper readies the longest-waiting special; story Entertainment District uses Gyutaro + Daki
- Tuned with the simulator; stats spreadsheet rebuilt from the roster

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -11,7 +11,7 @@
     <sheet name="HP % Calculator" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$S$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S59"/>
+  <dimension ref="A1:S69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="15" min="1" max="1"/>
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="26.85" customHeight="1" s="16">
+    <row r="3" ht="39.55" customHeight="1" s="16">
       <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Yoriichi (Age 85)</t>
@@ -818,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="16">
+    <row r="4" ht="26.85" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Muzan Kibutsuji (Final Form)</t>
@@ -962,7 +962,7 @@
       </c>
       <c r="S5" s="22" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1" s="16">
+    <row r="6" ht="26.85" customHeight="1" s="16">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Kokushibo</t>
@@ -1032,15 +1032,15 @@
       </c>
       <c r="S6" s="22" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="16">
+    <row r="7" ht="26.85" customHeight="1" s="16">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Doma</t>
+          <t>Tanjiro Kamado (Demon King)</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Demon King</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
@@ -1050,26 +1050,26 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 2</t>
+          <t>Demon King · Sun-proof</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H7" s="20" t="n">
         <v>11</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="21">
         <f>1/F7</f>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="P7" s="19" t="inlineStr">
         <is>
-          <t>Frozen Lotus</t>
+          <t>Demon King's Rampage</t>
         </is>
       </c>
       <c r="Q7" s="22" t="inlineStr">
@@ -1100,12 +1100,16 @@
       <c r="R7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S7" s="22" t="n"/>
+      <c r="S7" s="22" t="inlineStr">
+        <is>
+          <t>Sun-proof: Yoriichi's sun can't stop his regeneration. Still Tanjiro: Siblings, Kamaboko Squad and Mentor bonuses all apply.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="26.85" customHeight="1" s="16">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>Akaza</t>
+          <t>Doma</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
@@ -1120,26 +1124,26 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 3</t>
+          <t>Upper Moon 2</t>
         </is>
       </c>
       <c r="E8" s="20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F8" s="20" t="n">
         <v>44</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" s="21">
         <f>1/F8</f>
@@ -1159,12 +1163,12 @@
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Destructive Death</t>
+          <t>Frozen Lotus</t>
         </is>
       </c>
       <c r="Q8" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+6.</t>
+          <t>Every enemy takes PWR−4, ignores DEF.</t>
         </is>
       </c>
       <c r="R8" s="20" t="n">
@@ -1172,10 +1176,10 @@
       </c>
       <c r="S8" s="22" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="16">
+    <row r="9" ht="26.85" customHeight="1" s="16">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Hantengu</t>
+          <t>Akaza</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -1190,26 +1194,26 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 4</t>
+          <t>Upper Moon 3</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
         <v>9</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="21">
         <f>1/F9</f>
@@ -1229,27 +1233,23 @@
       </c>
       <c r="P9" s="19" t="inlineStr">
         <is>
-          <t>Cowering Hide</t>
+          <t>Destructive Death</t>
         </is>
       </c>
       <c r="Q9" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
+          <t>Strike for PWR+6.</t>
         </is>
       </c>
       <c r="R9" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S9" s="22" t="inlineStr">
-        <is>
-          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="16">
+      <c r="S9" s="22" t="n"/>
+    </row>
+    <row r="10" ht="26.85" customHeight="1" s="16">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>Gyokko</t>
+          <t>Hantengu</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -1264,26 +1264,26 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 5</t>
+          <t>Upper Moon 4</t>
         </is>
       </c>
       <c r="E10" s="20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I10" s="20" t="n">
         <v>4</v>
       </c>
       <c r="J10" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="21">
         <f>1/F10</f>
@@ -1303,28 +1303,32 @@
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>Water Prison Pot</t>
+          <t>Cowering Hide</t>
         </is>
       </c>
       <c r="Q10" s="22" t="inlineStr">
         <is>
-          <t>Traps one enemy: it takes PWR−2 (ignores DEF) and can't act next round.</t>
+          <t>Moves first. Hides: attacks miss him this round, and he heals 6.</t>
         </is>
       </c>
       <c r="R10" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S10" s="22" t="n"/>
+      <c r="S10" s="22" t="inlineStr">
+        <is>
+          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="26.85" customHeight="1" s="16">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Gyutaro &amp; Daki</t>
+          <t>Zohakuten</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Hatred</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1334,26 +1338,26 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6</t>
+          <t>Upper Moon 4 · Hatred</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I11" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="20" t="n">
-        <v>30</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="I11" s="20" t="n">
-        <v>4</v>
-      </c>
       <c r="J11" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" s="21">
         <f>1/F11</f>
@@ -1373,23 +1377,27 @@
       </c>
       <c r="P11" s="19" t="inlineStr">
         <is>
-          <t>Flying Blood Sickles</t>
+          <t>Wood Dragons</t>
         </is>
       </c>
       <c r="Q11" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
+          <t>Every enemy takes PWR−4, even through Defend.</t>
         </is>
       </c>
       <c r="R11" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S11" s="22" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="16">
+      <c r="S11" s="22" t="inlineStr">
+        <is>
+          <t>Hantengu's Hatred: his emotions merged into one body. He doesn't split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26.85" customHeight="1" s="16">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>Kaigaku</t>
+          <t>Gyokko</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
@@ -1404,26 +1412,26 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6 · fallen Thunder</t>
+          <t>Upper Moon 5</t>
         </is>
       </c>
       <c r="E12" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J12" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="21">
         <f>1/F12</f>
@@ -1443,27 +1451,23 @@
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>Black Thunder</t>
+          <t>Water Prison Pot</t>
         </is>
       </c>
       <c r="Q12" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3, and a second random enemy takes 4.</t>
+          <t>Traps one enemy: it takes PWR−2 (ignores DEF) and can't act next round.</t>
         </is>
       </c>
       <c r="R12" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S12" s="22" t="inlineStr">
-        <is>
-          <t>Rival: an enemy Zenitsu gets +2 PWR against him.</t>
-        </is>
-      </c>
+      <c r="S12" s="22" t="n"/>
     </row>
     <row r="13" ht="26.85" customHeight="1" s="16">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Enmu</t>
+          <t>Gyutaro</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -1478,26 +1482,26 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 1</t>
+          <t>Upper Moon 6</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G13" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H13" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I13" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="21">
         <f>1/F13</f>
@@ -1517,23 +1521,27 @@
       </c>
       <c r="P13" s="19" t="inlineStr">
         <is>
-          <t>Forced Sleep</t>
+          <t>Flying Blood Sickles</t>
         </is>
       </c>
       <c r="Q13" s="22" t="inlineStr">
         <is>
-          <t>Every enemy has to wait 2 more rounds for their special.</t>
+          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
         </is>
       </c>
       <c r="R13" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S13" s="22" t="n"/>
+      <c r="S13" s="22" t="inlineStr">
+        <is>
+          <t>Two as One: with Daki on his team he gets +2 PWR. If one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each). Knock both out in the same round to stop it.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26.85" customHeight="1" s="16">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Rui</t>
+          <t>Kaigaku</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -1548,23 +1556,23 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 5</t>
+          <t>Upper Moon 6 · fallen Thunder</t>
         </is>
       </c>
       <c r="E14" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J14" s="20" t="n">
         <v>1</v>
@@ -1587,23 +1595,27 @@
       </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>Cutting Thread Cage</t>
+          <t>Black Thunder</t>
         </is>
       </c>
       <c r="Q14" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR and stun the target next round.</t>
+          <t>Strike for PWR+3, and a second random enemy takes 4.</t>
         </is>
       </c>
       <c r="R14" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S14" s="22" t="n"/>
+      <c r="S14" s="22" t="inlineStr">
+        <is>
+          <t>Rival: an enemy Zenitsu gets +2 PWR against him.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="26.85" customHeight="1" s="16">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Kyogai</t>
+          <t>Daki</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
@@ -1618,26 +1630,26 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Former Lower Moon</t>
+          <t>Upper Moon 6</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I15" s="20" t="n">
         <v>3</v>
       </c>
       <c r="J15" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15" s="21">
         <f>1/F15</f>
@@ -1657,23 +1669,27 @@
       </c>
       <c r="P15" s="19" t="inlineStr">
         <is>
-          <t>Drum Room Spin</t>
+          <t>Obi Sashes</t>
         </is>
       </c>
       <c r="Q15" s="22" t="inlineStr">
         <is>
-          <t>Flip the room. The target is stunned next round.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R15" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="S15" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S15" s="22" t="inlineStr">
+        <is>
+          <t>Two as One: with Gyutaro on her team, if one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="26.85" customHeight="1" s="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>Swamp Demon</t>
+          <t>Enmu</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
@@ -1688,23 +1704,23 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Lesser demon</t>
+          <t>Lower Moon 1</t>
         </is>
       </c>
       <c r="E16" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H16" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" s="20" t="n">
         <v>1</v>
@@ -1727,23 +1743,23 @@
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Swamp Dive</t>
+          <t>Forced Sleep</t>
         </is>
       </c>
       <c r="Q16" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
+          <t>Every enemy has to wait 2 more rounds for their special.</t>
         </is>
       </c>
       <c r="R16" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" s="22" t="n"/>
     </row>
     <row r="17" ht="26.85" customHeight="1" s="16">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Hand Demon</t>
+          <t>Nakime</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
@@ -1758,26 +1774,26 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Final Selection</t>
+          <t>Upper Moon 4 · Infinity Castle</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I17" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="20" t="n">
         <v>2</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <v>14</v>
-      </c>
-      <c r="G17" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H17" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="J17" s="20" t="n">
-        <v>1</v>
       </c>
       <c r="K17" s="21">
         <f>1/F17</f>
@@ -1797,28 +1813,32 @@
       </c>
       <c r="P17" s="19" t="inlineStr">
         <is>
-          <t>Grasping Arms</t>
+          <t>Castle Shift</t>
         </is>
       </c>
       <c r="Q17" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Moves first. Sends an enemy to another room: they can't act and can't be hit this round.</t>
         </is>
       </c>
       <c r="R17" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S17" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S17" s="22" t="inlineStr">
+        <is>
+          <t>Biwa, not blade: she never attacks. Her basic move, Biwa Strum, makes an enemy act last this round. If she's the last one standing on her team, she flees and counts as knocked out.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="26.85" customHeight="1" s="16">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Sekido (Anger)</t>
+          <t>Rui</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
@@ -1828,23 +1848,23 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Anger</t>
+          <t>Lower Moon 5</t>
         </is>
       </c>
       <c r="E18" s="20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G18" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J18" s="20" t="n">
         <v>1</v>
@@ -1867,32 +1887,28 @@
       </c>
       <c r="P18" s="19" t="inlineStr">
         <is>
-          <t>Lightning Staff</t>
+          <t>Cutting Thread Cage</t>
         </is>
       </c>
       <c r="Q18" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4, ignores DEF.</t>
+          <t>Strike for PWR and stun the target next round.</t>
         </is>
       </c>
       <c r="R18" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S18" s="22" t="inlineStr">
-        <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="16">
+      <c r="S18" s="22" t="n"/>
+    </row>
+    <row r="19" ht="26.85" customHeight="1" s="16">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Karaku (Joy)</t>
+          <t>Yahaba</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
@@ -1902,20 +1918,20 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Joy</t>
+          <t>Arrow demon</t>
         </is>
       </c>
       <c r="E19" s="20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F19" s="20" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G19" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I19" s="20" t="n">
         <v>3</v>
@@ -1941,32 +1957,32 @@
       </c>
       <c r="P19" s="19" t="inlineStr">
         <is>
-          <t>Gale Fan</t>
+          <t>Vector Arrows</t>
         </is>
       </c>
       <c r="Q19" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Moves first. Bends an enemy's aim: every hit they throw this round misses.</t>
         </is>
       </c>
       <c r="R19" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S19" s="22" t="inlineStr">
         <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
+          <t>Temari &amp; Arrows: with Susamaru on his team, his arrows guide her hits past Defend.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26.85" customHeight="1" s="16">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Aizetsu (Sorrow)</t>
+          <t>Kyogai</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
@@ -1976,20 +1992,20 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Sorrow</t>
+          <t>Former Lower Moon</t>
         </is>
       </c>
       <c r="E20" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20" s="20" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H20" s="20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I20" s="20" t="n">
         <v>3</v>
@@ -2015,32 +2031,28 @@
       </c>
       <c r="P20" s="19" t="inlineStr">
         <is>
-          <t>Cross Spear</t>
+          <t>Drum Room Spin</t>
         </is>
       </c>
       <c r="Q20" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4.</t>
+          <t>Flip the room. The target is stunned next round.</t>
         </is>
       </c>
       <c r="R20" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S20" s="22" t="inlineStr">
-        <is>
-          <t>Appears when Sekido falls. Not drafted.</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="S20" s="22" t="n"/>
     </row>
     <row r="21" ht="26.85" customHeight="1" s="16">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Urogi (Pleasure)</t>
+          <t>Susamaru</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>Split form</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -2050,23 +2062,23 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Pleasure</t>
+          <t>Temari demon</t>
         </is>
       </c>
       <c r="E21" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="20" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="G21" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H21" s="20" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I21" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="20" t="n">
         <v>1</v>
@@ -2089,61 +2101,61 @@
       </c>
       <c r="P21" s="19" t="inlineStr">
         <is>
-          <t>Sky Dive</t>
+          <t>Temari Barrage</t>
         </is>
       </c>
       <c r="Q21" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Swoops down for PWR+2.</t>
+          <t>Strike your target and one other enemy for PWR−1.</t>
         </is>
       </c>
       <c r="R21" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S21" s="22" t="inlineStr">
+        <is>
+          <t>Temari &amp; Arrows: with Yahaba on her team, her hits slip past Defend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26.85" customHeight="1" s="16">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Swamp Demon</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>Demon</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Lesser demon</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I22" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="S21" s="22" t="inlineStr">
-        <is>
-          <t>Appears when Karaku falls. Not drafted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26.85" customHeight="1" s="16">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>Gyomei Himejima (Mark)</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>Slayer</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Stone Hashira</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="F22" s="20" t="n">
-        <v>50</v>
-      </c>
-      <c r="G22" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="H22" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I22" s="20" t="n">
-        <v>8</v>
-      </c>
       <c r="J22" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" s="21">
         <f>1/F22</f>
@@ -2163,61 +2175,57 @@
       </c>
       <c r="P22" s="19" t="inlineStr">
         <is>
-          <t>Volcanic Rock</t>
+          <t>Swamp Dive</t>
         </is>
       </c>
       <c r="Q22" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 11, ignores DEF.</t>
+          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
         </is>
       </c>
       <c r="R22" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="S22" s="22" t="inlineStr">
-        <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="16">
-      <c r="A23" s="23" t="inlineStr">
-        <is>
-          <t>Giyu Tomioka (Mark)</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+      <c r="S22" s="22" t="n"/>
+    </row>
+    <row r="23" ht="26.85" customHeight="1" s="16">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Hand Demon</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Water Hashira</t>
+          <t>Final Selection</t>
         </is>
       </c>
       <c r="E23" s="20" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F23" s="20" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G23" s="20" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H23" s="20" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I23" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J23" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="21">
         <f>1/F23</f>
@@ -2237,61 +2245,57 @@
       </c>
       <c r="P23" s="19" t="inlineStr">
         <is>
-          <t>Dead Calm</t>
+          <t>Grasping Arms</t>
         </is>
       </c>
       <c r="Q23" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Your whole team takes no damage this round.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R23" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S23" s="22" t="inlineStr">
-        <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="16">
-      <c r="A24" s="23" t="inlineStr">
-        <is>
-          <t>Muichiro Tokito (Mark)</t>
-        </is>
-      </c>
-      <c r="B24" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+        <v>2</v>
+      </c>
+      <c r="S23" s="22" t="n"/>
+    </row>
+    <row r="24" ht="26.85" customHeight="1" s="16">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Aizetsu (Sorrow)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Mist Hashira</t>
+          <t>Hantengu split · Sorrow</t>
         </is>
       </c>
       <c r="E24" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="F24" s="20" t="n">
-        <v>34</v>
-      </c>
       <c r="G24" s="20" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H24" s="20" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="I24" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J24" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" s="21">
         <f>1/F24</f>
@@ -2311,61 +2315,61 @@
       </c>
       <c r="P24" s="19" t="inlineStr">
         <is>
-          <t>Obscuring Clouds</t>
+          <t>Cross Spear</t>
         </is>
       </c>
       <c r="Q24" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
+          <t>Strike for PWR+4.</t>
         </is>
       </c>
       <c r="R24" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S24" s="22" t="inlineStr">
         <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="16">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>Sanemi Shinazugawa (Mark)</t>
-        </is>
-      </c>
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>Mark</t>
+          <t>Appears when Sekido falls. Not drafted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26.85" customHeight="1" s="16">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Karaku (Joy)</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Wind Hashira</t>
+          <t>Hantengu split · Joy</t>
         </is>
       </c>
       <c r="E25" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H25" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="F25" s="20" t="n">
-        <v>42</v>
-      </c>
-      <c r="G25" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="H25" s="20" t="n">
-        <v>11</v>
-      </c>
       <c r="I25" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J25" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" s="21">
         <f>1/F25</f>
@@ -2385,12 +2389,12 @@
       </c>
       <c r="P25" s="19" t="inlineStr">
         <is>
-          <t>Black Wind Mountain Mist</t>
+          <t>Gale Fan</t>
         </is>
       </c>
       <c r="Q25" s="22" t="inlineStr">
         <is>
-          <t>Strike your target and one other enemy for PWR.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R25" s="20" t="n">
@@ -2398,48 +2402,48 @@
       </c>
       <c r="S25" s="22" t="inlineStr">
         <is>
-          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="16">
+          <t>Appears when Hantengu falls. Not drafted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26.85" customHeight="1" s="16">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Giyu Tomioka</t>
+          <t>Sekido (Anger)</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Water Hashira</t>
+          <t>Hantengu split · Anger</t>
         </is>
       </c>
       <c r="E26" s="20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H26" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I26" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J26" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" s="21">
         <f>1/F26</f>
@@ -2459,57 +2463,61 @@
       </c>
       <c r="P26" s="19" t="inlineStr">
         <is>
-          <t>Dead Calm</t>
+          <t>Lightning Staff</t>
         </is>
       </c>
       <c r="Q26" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Your whole team takes no damage this round.</t>
+          <t>Every enemy takes 4, ignores DEF.</t>
         </is>
       </c>
       <c r="R26" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="S26" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S26" s="22" t="inlineStr">
+        <is>
+          <t>Appears when Hantengu falls. Not drafted.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="26.85" customHeight="1" s="16">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>Gyomei Himejima</t>
+          <t>Urogi (Pleasure)</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Stone Hashira</t>
+          <t>Hantengu split · Pleasure</t>
         </is>
       </c>
       <c r="E27" s="20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F27" s="20" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="G27" s="20" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H27" s="20" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I27" s="20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J27" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="21">
         <f>1/F27</f>
@@ -2529,23 +2537,27 @@
       </c>
       <c r="P27" s="19" t="inlineStr">
         <is>
-          <t>Volcanic Rock</t>
+          <t>Sky Dive</t>
         </is>
       </c>
       <c r="Q27" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 9, ignores DEF.</t>
+          <t>Moves early. Swoops down for PWR+2.</t>
         </is>
       </c>
       <c r="R27" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S27" s="22" t="n"/>
-    </row>
-    <row r="28" ht="39.55" customHeight="1" s="16">
+        <v>2</v>
+      </c>
+      <c r="S27" s="22" t="inlineStr">
+        <is>
+          <t>Appears when Karaku falls. Not drafted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26.85" customHeight="1" s="16">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Mitsuri Kanroji (Mark)</t>
+          <t>Gyomei Himejima (Mark)</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
@@ -2560,23 +2572,23 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Love Hashira</t>
+          <t>Stone Hashira</t>
         </is>
       </c>
       <c r="E28" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" s="20" t="n">
         <v>8</v>
-      </c>
-      <c r="F28" s="20" t="n">
-        <v>36</v>
-      </c>
-      <c r="G28" s="20" t="n">
-        <v>13</v>
-      </c>
-      <c r="H28" s="20" t="n">
-        <v>11</v>
-      </c>
-      <c r="I28" s="20" t="n">
-        <v>5</v>
       </c>
       <c r="J28" s="20" t="n">
         <v>0</v>
@@ -2599,12 +2611,12 @@
       </c>
       <c r="P28" s="19" t="inlineStr">
         <is>
-          <t>Catlove Shower</t>
+          <t>Volcanic Rock</t>
         </is>
       </c>
       <c r="Q28" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Every enemy takes 11, ignoring DEF.</t>
         </is>
       </c>
       <c r="R28" s="20" t="n">
@@ -2616,10 +2628,10 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="16">
+    <row r="29" ht="26.85" customHeight="1" s="16">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t>Obanai Iguro (Mark)</t>
+          <t>Giyu Tomioka (Mark)</t>
         </is>
       </c>
       <c r="B29" s="23" t="inlineStr">
@@ -2634,23 +2646,23 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Serpent Hashira</t>
+          <t>Water Hashira</t>
         </is>
       </c>
       <c r="E29" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F29" s="20" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G29" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H29" s="20" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I29" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29" s="20" t="n">
         <v>0</v>
@@ -2673,16 +2685,16 @@
       </c>
       <c r="P29" s="19" t="inlineStr">
         <is>
-          <t>Twin-Headed Reptile</t>
+          <t>Dead Calm</t>
         </is>
       </c>
       <c r="Q29" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
+          <t>Moves first. Your whole team takes no damage this round.</t>
         </is>
       </c>
       <c r="R29" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S29" s="22" t="inlineStr">
         <is>
@@ -2690,10 +2702,10 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="16">
+    <row r="30" ht="26.85" customHeight="1" s="16">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>Tanjiro Kamado (Mark)</t>
+          <t>Muichiro Tokito (Mark)</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
@@ -2708,20 +2720,20 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Sun &amp; Water</t>
+          <t>Mist Hashira</t>
         </is>
       </c>
       <c r="E30" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30" s="20" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G30" s="20" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H30" s="20" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I30" s="20" t="n">
         <v>5</v>
@@ -2747,12 +2759,12 @@
       </c>
       <c r="P30" s="19" t="inlineStr">
         <is>
-          <t>Hinokami Kagura</t>
+          <t>Obscuring Clouds</t>
         </is>
       </c>
       <c r="Q30" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+5, ignores DEF.</t>
+          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
         </is>
       </c>
       <c r="R30" s="20" t="n">
@@ -2764,15 +2776,15 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="16">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Kyojuro Rengoku</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+    <row r="31" ht="26.85" customHeight="1" s="16">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>Sanemi Shinazugawa (Mark)</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
@@ -2782,23 +2794,23 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Flame Hashira</t>
+          <t>Wind Hashira</t>
         </is>
       </c>
       <c r="E31" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F31" s="20" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G31" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="H31" s="20" t="n">
-        <v>9</v>
-      </c>
       <c r="I31" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J31" s="20" t="n">
         <v>0</v>
@@ -2821,57 +2833,61 @@
       </c>
       <c r="P31" s="19" t="inlineStr">
         <is>
-          <t>Ninth Form: Rengoku</t>
+          <t>Black Wind Mountain Mist</t>
         </is>
       </c>
       <c r="Q31" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+8.</t>
+          <t>Strike your target and one other enemy for PWR.</t>
         </is>
       </c>
       <c r="R31" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S31" s="22" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="16">
+        <v>2</v>
+      </c>
+      <c r="S31" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26.85" customHeight="1" s="16">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>Muichiro Tokito</t>
+          <t>Nezuko Kamado (Awakened)</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Awakened</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Mist Hashira</t>
+          <t>Demon ally · Awakened</t>
         </is>
       </c>
       <c r="E32" s="20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G32" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="H32" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="H32" s="20" t="n">
-        <v>11</v>
-      </c>
       <c r="I32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J32" s="20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K32" s="21">
         <f>1/F32</f>
@@ -2891,23 +2907,27 @@
       </c>
       <c r="P32" s="19" t="inlineStr">
         <is>
-          <t>Obscuring Clouds</t>
+          <t>Exploding Blood</t>
         </is>
       </c>
       <c r="Q32" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
+          <t>Every enemy takes 10, ignores DEF, and poison burns off your whole team.</t>
         </is>
       </c>
       <c r="R32" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S32" s="22" t="n"/>
+      <c r="S32" s="22" t="inlineStr">
+        <is>
+          <t>Berserk: she can't Defend.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="26.85" customHeight="1" s="16">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>Sanemi Shinazugawa</t>
+          <t>Giyu Tomioka</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -2922,20 +2942,20 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Wind Hashira</t>
+          <t>Water Hashira</t>
         </is>
       </c>
       <c r="E33" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F33" s="20" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G33" s="20" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H33" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I33" s="20" t="n">
         <v>5</v>
@@ -2961,23 +2981,23 @@
       </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
-          <t>Black Wind Mountain Mist</t>
+          <t>Dead Calm</t>
         </is>
       </c>
       <c r="Q33" s="22" t="inlineStr">
         <is>
-          <t>Strike your target and one other enemy for PWR.</t>
+          <t>Moves first. Your whole team takes no damage this round.</t>
         </is>
       </c>
       <c r="R33" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S33" s="22" t="n"/>
     </row>
-    <row r="34" ht="15" customHeight="1" s="16">
+    <row r="34" ht="26.85" customHeight="1" s="16">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>Tengen Uzui</t>
+          <t>Gyomei Himejima</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -2992,23 +3012,23 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Sound Hashira</t>
+          <t>Stone Hashira</t>
         </is>
       </c>
       <c r="E34" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H34" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I34" s="20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J34" s="20" t="n">
         <v>0</v>
@@ -3031,12 +3051,12 @@
       </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
-          <t>Constant Resounding Slashes</t>
+          <t>Volcanic Rock</t>
         </is>
       </c>
       <c r="Q34" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−2.</t>
+          <t>Every enemy takes 9, ignoring DEF.</t>
         </is>
       </c>
       <c r="R34" s="20" t="n">
@@ -3045,14 +3065,14 @@
       <c r="S34" s="22" t="n"/>
     </row>
     <row r="35" ht="26.85" customHeight="1" s="16">
-      <c r="A35" s="19" t="inlineStr">
-        <is>
-          <t>Mitsuri Kanroji</t>
-        </is>
-      </c>
-      <c r="B35" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>Mitsuri Kanroji (Mark)</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
@@ -3066,19 +3086,19 @@
         </is>
       </c>
       <c r="E35" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <v>36</v>
+      </c>
+      <c r="G35" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="H35" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I35" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F35" s="20" t="n">
-        <v>28</v>
-      </c>
-      <c r="G35" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="H35" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="I35" s="20" t="n">
-        <v>4</v>
       </c>
       <c r="J35" s="20" t="n">
         <v>0</v>
@@ -3110,19 +3130,23 @@
         </is>
       </c>
       <c r="R35" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S35" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S35" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26.85" customHeight="1" s="16">
-      <c r="A36" s="19" t="inlineStr">
-        <is>
-          <t>Obanai Iguro</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Obanai Iguro (Mark)</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
@@ -3136,19 +3160,19 @@
         </is>
       </c>
       <c r="E36" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F36" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="G36" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="H36" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="I36" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F36" s="20" t="n">
-        <v>26</v>
-      </c>
-      <c r="G36" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="H36" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I36" s="20" t="n">
-        <v>4</v>
       </c>
       <c r="J36" s="20" t="n">
         <v>0</v>
@@ -3180,19 +3204,23 @@
         </is>
       </c>
       <c r="R36" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S36" s="22" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="S36" s="22" t="inlineStr">
+        <is>
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="26.85" customHeight="1" s="16">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>Shinobu Kocho</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>Base</t>
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>Tanjiro Kamado (Mark)</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
@@ -3202,23 +3230,23 @@
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Insect Hashira</t>
+          <t>Sun &amp; Water</t>
         </is>
       </c>
       <c r="E37" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <v>36</v>
+      </c>
+      <c r="G37" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="H37" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I37" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F37" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="G37" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J37" s="20" t="n">
         <v>0</v>
@@ -3241,27 +3269,27 @@
       </c>
       <c r="P37" s="19" t="inlineStr">
         <is>
-          <t>Wisteria Poison</t>
+          <t>Hinokami Kagura</t>
         </is>
       </c>
       <c r="Q37" s="22" t="inlineStr">
         <is>
-          <t>Poison a target for 3 rounds: 6/round to demons, 3/round to humans.</t>
+          <t>Strike for PWR+5, ignores DEF.</t>
         </is>
       </c>
       <c r="R37" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S37" s="22" t="inlineStr">
         <is>
-          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match. (Not Akaza: he never eats women.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+          <t>Mark awakened: boosted stats and the special recharges 1 round faster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26.85" customHeight="1" s="16">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>Tanjiro Kamado</t>
+          <t>Kyojuro Rengoku</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -3276,23 +3304,23 @@
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Sun &amp; Water</t>
+          <t>Flame Hashira</t>
         </is>
       </c>
       <c r="E38" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="F38" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="G38" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="H38" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I38" s="20" t="n">
         <v>5</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>28</v>
-      </c>
-      <c r="G38" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="H38" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v>4</v>
       </c>
       <c r="J38" s="20" t="n">
         <v>0</v>
@@ -3315,12 +3343,12 @@
       </c>
       <c r="P38" s="19" t="inlineStr">
         <is>
-          <t>Hinokami Kagura</t>
+          <t>Ninth Form: Rengoku</t>
         </is>
       </c>
       <c r="Q38" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+5, ignores DEF.</t>
+          <t>Strike for PWR+8.</t>
         </is>
       </c>
       <c r="R38" s="20" t="n">
@@ -3328,10 +3356,10 @@
       </c>
       <c r="S38" s="22" t="n"/>
     </row>
-    <row r="39" ht="15" customHeight="1" s="16">
+    <row r="39" ht="26.85" customHeight="1" s="16">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>Inosuke Hashibira</t>
+          <t>Muichiro Tokito</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -3346,23 +3374,23 @@
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Beast</t>
+          <t>Mist Hashira</t>
         </is>
       </c>
       <c r="E39" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="G39" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H39" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I39" s="20" t="n">
         <v>4</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>28</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="H39" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="I39" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J39" s="20" t="n">
         <v>0</v>
@@ -3385,23 +3413,23 @@
       </c>
       <c r="P39" s="19" t="inlineStr">
         <is>
-          <t>Fang Frenzy</t>
+          <t>Obscuring Clouds</t>
         </is>
       </c>
       <c r="Q39" s="22" t="inlineStr">
         <is>
-          <t>Two wild strikes of PWR−1 at random enemies.</t>
+          <t>Moves early. Vanishes into mist (attacks miss him this round) and strikes for PWR+2.</t>
         </is>
       </c>
       <c r="R39" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S39" s="22" t="n"/>
     </row>
-    <row r="40" ht="15" customHeight="1" s="16">
+    <row r="40" ht="26.85" customHeight="1" s="16">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>Kanao Tsuyuri</t>
+          <t>Sanemi Shinazugawa</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -3416,23 +3444,23 @@
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Flower</t>
+          <t>Wind Hashira</t>
         </is>
       </c>
       <c r="E40" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G40" s="20" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H40" s="20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I40" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J40" s="20" t="n">
         <v>0</v>
@@ -3455,12 +3483,12 @@
       </c>
       <c r="P40" s="19" t="inlineStr">
         <is>
-          <t>Equinoctial Vermilion Eye</t>
+          <t>Black Wind Mountain Mist</t>
         </is>
       </c>
       <c r="Q40" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Strike for PWR+4.</t>
+          <t>Strike your target and one other enemy for PWR.</t>
         </is>
       </c>
       <c r="R40" s="20" t="n">
@@ -3468,10 +3496,10 @@
       </c>
       <c r="S40" s="22" t="n"/>
     </row>
-    <row r="41" ht="15" customHeight="1" s="16">
+    <row r="41" ht="26.85" customHeight="1" s="16">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>Nezuko Kamado</t>
+          <t>Tengen Uzui</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -3481,31 +3509,31 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Sound Hashira</t>
         </is>
       </c>
       <c r="E41" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F41" s="20" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G41" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H41" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I41" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J41" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" s="21">
         <f>1/F41</f>
@@ -3525,12 +3553,12 @@
       </c>
       <c r="P41" s="19" t="inlineStr">
         <is>
-          <t>Exploding Blood</t>
+          <t>Constant Resounding Slashes</t>
         </is>
       </c>
       <c r="Q41" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 5, ignores DEF.</t>
+          <t>Every enemy takes PWR−2.</t>
         </is>
       </c>
       <c r="R41" s="20" t="n">
@@ -3538,10 +3566,10 @@
       </c>
       <c r="S41" s="22" t="n"/>
     </row>
-    <row r="42" ht="15" customHeight="1" s="16">
+    <row r="42" ht="26.85" customHeight="1" s="16">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>Sabito &amp; Makomo</t>
+          <t>Kanae Kocho</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -3556,23 +3584,23 @@
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>Spirits · Urokodaki's students</t>
+          <t>Former Flower Hashira</t>
         </is>
       </c>
       <c r="E42" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G42" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="H42" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I42" s="20" t="n">
         <v>4</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="H42" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I42" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J42" s="20" t="n">
         <v>0</v>
@@ -3595,12 +3623,12 @@
       </c>
       <c r="P42" s="19" t="inlineStr">
         <is>
-          <t>Spirit Training</t>
+          <t>Crimson Hanagoromo</t>
         </is>
       </c>
       <c r="Q42" s="22" t="inlineStr">
         <is>
-          <t>Train an ally (or themselves): +2 PWR for the rest of the match.</t>
+          <t>Strike for PWR+3, and your most hurt fighter heals 4.</t>
         </is>
       </c>
       <c r="R42" s="20" t="n">
@@ -3608,14 +3636,14 @@
       </c>
       <c r="S42" s="22" t="inlineStr">
         <is>
-          <t>Urokodaki's students: they get his Mentor bonus too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
+          <t>Retired: she no longer counts as a Hashira. Kocho Sisters: with Shinobu on her team, Shinobu's poison lasts a round longer. Her student Kanao gets +1 PWR on her team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26.85" customHeight="1" s="16">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>Sakonji Urokodaki</t>
+          <t>Mitsuri Kanroji</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -3630,20 +3658,20 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Former Water Hashira</t>
+          <t>Love Hashira</t>
         </is>
       </c>
       <c r="E43" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F43" s="20" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G43" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H43" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I43" s="20" t="n">
         <v>4</v>
@@ -3669,32 +3697,28 @@
       </c>
       <c r="P43" s="19" t="inlineStr">
         <is>
-          <t>Water Wheel</t>
+          <t>Catlove Shower</t>
         </is>
       </c>
       <c r="Q43" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R43" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S43" s="22" t="inlineStr">
-        <is>
-          <t>Mentor: Tanjiro, Giyu and Sabito &amp; Makomo on his team get +1 DEF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
+        <v>3</v>
+      </c>
+      <c r="S43" s="22" t="n"/>
+    </row>
+    <row r="44" ht="26.85" customHeight="1" s="16">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>Tengen Uzui (Retired)</t>
+          <t>Obanai Iguro</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Retired</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
@@ -3704,20 +3728,20 @@
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>Former Sound Hashira</t>
+          <t>Serpent Hashira</t>
         </is>
       </c>
       <c r="E44" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G44" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H44" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I44" s="20" t="n">
         <v>4</v>
@@ -3743,27 +3767,23 @@
       </c>
       <c r="P44" s="19" t="inlineStr">
         <is>
-          <t>Bodyguard</t>
+          <t>Twin-Headed Reptile</t>
         </is>
       </c>
       <c r="Q44" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Shields an ally (or himself): they count as Defending this round and take half damage.</t>
+          <t>Strike for PWR+4. Slips past guards (Defend does nothing).</t>
         </is>
       </c>
       <c r="R44" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S44" s="22" t="inlineStr">
-        <is>
-          <t>Retired: lost a hand and an eye, so he no longer counts as a Hashira.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
+        <v>3</v>
+      </c>
+      <c r="S44" s="22" t="n"/>
+    </row>
+    <row r="45" ht="26.85" customHeight="1" s="16">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>Zenitsu Agatsuma</t>
+          <t>Shinobu Kocho</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -3778,23 +3798,23 @@
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Thunder</t>
+          <t>Insect Hashira</t>
         </is>
       </c>
       <c r="E45" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F45" s="20" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G45" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H45" s="20" t="n">
         <v>10</v>
       </c>
       <c r="I45" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J45" s="20" t="n">
         <v>0</v>
@@ -3817,23 +3837,27 @@
       </c>
       <c r="P45" s="19" t="inlineStr">
         <is>
-          <t>Thunderclap and Flash</t>
+          <t>Wisteria Poison</t>
         </is>
       </c>
       <c r="Q45" s="22" t="inlineStr">
         <is>
-          <t>Always moves first. Strike for PWR×2.</t>
+          <t>Poison a target for 3 rounds: 6/round to demons, 3/round to humans.</t>
         </is>
       </c>
       <c r="R45" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S45" s="22" t="n"/>
-    </row>
-    <row r="46">
+      <c r="S45" s="22" t="inlineStr">
+        <is>
+          <t>Wisteria Body: if a demon lands the blow that knocks her out, it devours her and loses 5 HP every round for the rest of the match. (Not Akaza: he never eats women.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26.85" customHeight="1" s="16">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Genya Shinazugawa</t>
+          <t>Tanjiro Kamado</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -3848,23 +3872,23 @@
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>Demon eater</t>
+          <t>Sun &amp; Water</t>
         </is>
       </c>
       <c r="E46" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F46" s="20" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G46" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H46" s="20" t="n">
         <v>7</v>
       </c>
       <c r="I46" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J46" s="20" t="n">
         <v>0</v>
@@ -3887,12 +3911,12 @@
       </c>
       <c r="P46" s="19" t="inlineStr">
         <is>
-          <t>Demon Consumption</t>
+          <t>Hinokami Kagura</t>
         </is>
       </c>
       <c r="Q46" s="22" t="inlineStr">
         <is>
-          <t>Heal 8 and gain +2 PWR for the rest of the match.</t>
+          <t>Strike for PWR+5, ignores DEF.</t>
         </is>
       </c>
       <c r="R46" s="20" t="n">
@@ -3900,10 +3924,10 @@
       </c>
       <c r="S46" s="22" t="n"/>
     </row>
-    <row r="47">
+    <row r="47" ht="26.85" customHeight="1" s="16">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Tamayo</t>
+          <t>Genya Shinazugawa</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -3913,22 +3937,22 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Physician · Demon ally</t>
+          <t>Demon eater</t>
         </is>
       </c>
       <c r="E47" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F47" s="20" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G47" s="20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H47" s="20" t="n">
         <v>7</v>
@@ -3937,7 +3961,7 @@
         <v>3</v>
       </c>
       <c r="J47" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K47" s="21">
         <f>1/F47</f>
@@ -3957,27 +3981,23 @@
       </c>
       <c r="P47" s="19" t="inlineStr">
         <is>
-          <t>Healing Blood Art</t>
+          <t>Demon Consumption</t>
         </is>
       </c>
       <c r="Q47" s="22" t="inlineStr">
         <is>
-          <t>Heal an ally (or herself) for 10 and cure poison.</t>
+          <t>Heal 8 and gain +2 PWR for the rest of the match.</t>
         </is>
       </c>
       <c r="R47" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S47" s="22" t="inlineStr">
-        <is>
-          <t>Anti-Muzan Medicine: an enemy Muzan's regeneration drops by 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
+        <v>3</v>
+      </c>
+      <c r="S47" s="22" t="n"/>
+    </row>
+    <row r="48" ht="26.85" customHeight="1" s="16">
       <c r="A48" s="19" t="inlineStr">
         <is>
-          <t>Yushiro</t>
+          <t>Inosuke Hashibira</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -3987,31 +4007,31 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Demon ally</t>
+          <t>Slayer</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>Tamayo's guardian · Demon ally</t>
+          <t>Beast</t>
         </is>
       </c>
       <c r="E48" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G48" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H48" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I48" s="20" t="n">
         <v>3</v>
       </c>
       <c r="J48" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" s="21">
         <f>1/F48</f>
@@ -4031,23 +4051,23 @@
       </c>
       <c r="P48" s="19" t="inlineStr">
         <is>
-          <t>Concealment Talisman</t>
+          <t>Fang Frenzy</t>
         </is>
       </c>
       <c r="Q48" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Hide an ally (or himself): attacks against them miss this round.</t>
+          <t>Two wild strikes of PWR−1 at random enemies.</t>
         </is>
       </c>
       <c r="R48" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S48" s="22" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="26.85" customHeight="1" s="16">
       <c r="A49" s="19" t="inlineStr">
         <is>
-          <t>Kagaya Ubuyashiki</t>
+          <t>Kanao Tsuyuri</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -4062,23 +4082,23 @@
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Corps Master</t>
+          <t>Flower</t>
         </is>
       </c>
       <c r="E49" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F49" s="20" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G49" s="20" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H49" s="20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I49" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49" s="20" t="n">
         <v>0</v>
@@ -4101,27 +4121,23 @@
       </c>
       <c r="P49" s="19" t="inlineStr">
         <is>
-          <t>Words of Resolve</t>
+          <t>Equinoctial Vermilion Eye</t>
         </is>
       </c>
       <c r="Q49" s="22" t="inlineStr">
         <is>
-          <t>Every ally, himself included, heals 4.</t>
+          <t>Moves early. Strike for PWR+4.</t>
         </is>
       </c>
       <c r="R49" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S49" s="22" t="inlineStr">
-        <is>
-          <t>Master of the Corps: every Hashira on his team gets +1 DEF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
+      <c r="S49" s="22" t="n"/>
+    </row>
+    <row r="50" ht="26.85" customHeight="1" s="16">
       <c r="A50" s="19" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Nezuko Kamado</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -4131,31 +4147,31 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Slayer</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>Water · rank and file</t>
+          <t>Demon ally</t>
         </is>
       </c>
       <c r="E50" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F50" s="20" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G50" s="20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H50" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I50" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J50" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K50" s="21">
         <f>1/F50</f>
@@ -4175,214 +4191,919 @@
       </c>
       <c r="P50" s="19" t="inlineStr">
         <is>
+          <t>Exploding Blood</t>
+        </is>
+      </c>
+      <c r="Q50" s="22" t="inlineStr">
+        <is>
+          <t>Every enemy takes 5, ignores DEF.</t>
+        </is>
+      </c>
+      <c r="R50" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S50" s="22" t="n"/>
+    </row>
+    <row r="51" ht="26.85" customHeight="1" s="16">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>Sabito &amp; Makomo</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Spirits · Urokodaki's students</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="G51" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H51" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J51" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="21">
+        <f>1/F51</f>
+        <v/>
+      </c>
+      <c r="L51" s="21">
+        <f>J51/F51</f>
+        <v/>
+      </c>
+      <c r="M51" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" s="20" t="n"/>
+      <c r="O51" s="21">
+        <f>IF(N51="","",N51/F51)</f>
+        <v/>
+      </c>
+      <c r="P51" s="19" t="inlineStr">
+        <is>
+          <t>Spirit Training</t>
+        </is>
+      </c>
+      <c r="Q51" s="22" t="inlineStr">
+        <is>
+          <t>Train an ally (or themselves): +2 PWR for the rest of the match.</t>
+        </is>
+      </c>
+      <c r="R51" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S51" s="22" t="inlineStr">
+        <is>
+          <t>Urokodaki's students: they get his Mentor bonus too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="26.85" customHeight="1" s="16">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>Sakonji Urokodaki</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>Former Water Hashira</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F52" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="G52" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H52" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I52" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J52" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="21">
+        <f>1/F52</f>
+        <v/>
+      </c>
+      <c r="L52" s="21">
+        <f>J52/F52</f>
+        <v/>
+      </c>
+      <c r="M52" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="20" t="n"/>
+      <c r="O52" s="21">
+        <f>IF(N52="","",N52/F52)</f>
+        <v/>
+      </c>
+      <c r="P52" s="19" t="inlineStr">
+        <is>
+          <t>Water Wheel</t>
+        </is>
+      </c>
+      <c r="Q52" s="22" t="inlineStr">
+        <is>
+          <t>Strike for PWR+3.</t>
+        </is>
+      </c>
+      <c r="R52" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="S52" s="22" t="inlineStr">
+        <is>
+          <t>Mentor: Tanjiro, Giyu and Sabito &amp; Makomo on his team get +1 DEF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="26.85" customHeight="1" s="16">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>Tengen Uzui (Retired)</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>Former Sound Hashira</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G53" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H53" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I53" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J53" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="21">
+        <f>1/F53</f>
+        <v/>
+      </c>
+      <c r="L53" s="21">
+        <f>J53/F53</f>
+        <v/>
+      </c>
+      <c r="M53" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" s="20" t="n"/>
+      <c r="O53" s="21">
+        <f>IF(N53="","",N53/F53)</f>
+        <v/>
+      </c>
+      <c r="P53" s="19" t="inlineStr">
+        <is>
+          <t>Bodyguard</t>
+        </is>
+      </c>
+      <c r="Q53" s="22" t="inlineStr">
+        <is>
+          <t>Moves first. Shields an ally (or himself): they count as Defending this round and take half damage.</t>
+        </is>
+      </c>
+      <c r="R53" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="S53" s="22" t="inlineStr">
+        <is>
+          <t>Retired: lost a hand and an eye, so he no longer counts as a Hashira.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26.85" customHeight="1" s="16">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>Yoriichi Type Zero</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t>Puppet</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>Training puppet</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F54" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="G54" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I54" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J54" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="21">
+        <f>1/F54</f>
+        <v/>
+      </c>
+      <c r="L54" s="21">
+        <f>J54/F54</f>
+        <v/>
+      </c>
+      <c r="M54" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" s="20" t="n"/>
+      <c r="O54" s="21">
+        <f>IF(N54="","",N54/F54)</f>
+        <v/>
+      </c>
+      <c r="P54" s="19" t="inlineStr">
+        <is>
+          <t>Training Drill</t>
+        </is>
+      </c>
+      <c r="Q54" s="22" t="inlineStr">
+        <is>
+          <t>Drill an ally (or itself): +2 SPD for the rest of the match.</t>
+        </is>
+      </c>
+      <c r="R54" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S54" s="22" t="inlineStr">
+        <is>
+          <t>Six Arms: strikes three times every Attack. Only a puppet: it doesn't count as Yoriichi, so Muzan isn't scared of it. Training partner: Muichiro gets +1 PWR on its team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="26.85" customHeight="1" s="16">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>Zenitsu Agatsuma</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Thunder</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H55" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="I55" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="21">
+        <f>1/F55</f>
+        <v/>
+      </c>
+      <c r="L55" s="21">
+        <f>J55/F55</f>
+        <v/>
+      </c>
+      <c r="M55" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" s="20" t="n"/>
+      <c r="O55" s="21">
+        <f>IF(N55="","",N55/F55)</f>
+        <v/>
+      </c>
+      <c r="P55" s="19" t="inlineStr">
+        <is>
+          <t>Thunderclap and Flash</t>
+        </is>
+      </c>
+      <c r="Q55" s="22" t="inlineStr">
+        <is>
+          <t>Always moves first. Strike for PWR×2.</t>
+        </is>
+      </c>
+      <c r="R55" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S55" s="22" t="n"/>
+    </row>
+    <row r="56" ht="26.85" customHeight="1" s="16">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>Tamayo</t>
+        </is>
+      </c>
+      <c r="B56" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>Demon ally</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>Physician · Demon ally</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="G56" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H56" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I56" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J56" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="21">
+        <f>1/F56</f>
+        <v/>
+      </c>
+      <c r="L56" s="21">
+        <f>J56/F56</f>
+        <v/>
+      </c>
+      <c r="M56" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" s="20" t="n"/>
+      <c r="O56" s="21">
+        <f>IF(N56="","",N56/F56)</f>
+        <v/>
+      </c>
+      <c r="P56" s="19" t="inlineStr">
+        <is>
+          <t>Healing Blood Art</t>
+        </is>
+      </c>
+      <c r="Q56" s="22" t="inlineStr">
+        <is>
+          <t>Heal an ally (or herself) for 10 and cure poison.</t>
+        </is>
+      </c>
+      <c r="R56" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="S56" s="22" t="inlineStr">
+        <is>
+          <t>Anti-Muzan Medicine: an enemy Muzan's regeneration drops by 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="26.85" customHeight="1" s="16">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>Yushiro</t>
+        </is>
+      </c>
+      <c r="B57" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>Demon ally</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Tamayo's guardian · Demon ally</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="G57" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H57" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I57" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J57" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="21">
+        <f>1/F57</f>
+        <v/>
+      </c>
+      <c r="L57" s="21">
+        <f>J57/F57</f>
+        <v/>
+      </c>
+      <c r="M57" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" s="20" t="n"/>
+      <c r="O57" s="21">
+        <f>IF(N57="","",N57/F57)</f>
+        <v/>
+      </c>
+      <c r="P57" s="19" t="inlineStr">
+        <is>
+          <t>Concealment Talisman</t>
+        </is>
+      </c>
+      <c r="Q57" s="22" t="inlineStr">
+        <is>
+          <t>Moves first. Hide an ally (or himself): attacks against them miss this round.</t>
+        </is>
+      </c>
+      <c r="R57" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S57" s="22" t="n"/>
+    </row>
+    <row r="58" ht="26.85" customHeight="1" s="16">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>Kagaya Ubuyashiki</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C58" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D58" s="19" t="inlineStr">
+        <is>
+          <t>Corps Master</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F58" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="G58" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I58" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="21">
+        <f>1/F58</f>
+        <v/>
+      </c>
+      <c r="L58" s="21">
+        <f>J58/F58</f>
+        <v/>
+      </c>
+      <c r="M58" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" s="20" t="n"/>
+      <c r="O58" s="21">
+        <f>IF(N58="","",N58/F58)</f>
+        <v/>
+      </c>
+      <c r="P58" s="19" t="inlineStr">
+        <is>
+          <t>Words of Resolve</t>
+        </is>
+      </c>
+      <c r="Q58" s="22" t="inlineStr">
+        <is>
+          <t>Every ally, himself included, heals 4.</t>
+        </is>
+      </c>
+      <c r="R58" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S58" s="22" t="inlineStr">
+        <is>
+          <t>Master of the Corps: every Hashira on his team gets +1 DEF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="26.85" customHeight="1" s="16">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>Murata</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Slayer</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Water · rank and file</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G59" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H59" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="I59" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="J59" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="21">
+        <f>1/F59</f>
+        <v/>
+      </c>
+      <c r="L59" s="21">
+        <f>J59/F59</f>
+        <v/>
+      </c>
+      <c r="M59" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" s="20" t="n"/>
+      <c r="O59" s="21">
+        <f>IF(N59="","",N59/F59)</f>
+        <v/>
+      </c>
+      <c r="P59" s="19" t="inlineStr">
+        <is>
           <t>Water Surface Slash</t>
         </is>
       </c>
-      <c r="Q50" s="22" t="inlineStr">
+      <c r="Q59" s="22" t="inlineStr">
         <is>
           <t>Strike for PWR+2.</t>
         </is>
       </c>
-      <c r="R50" s="20" t="n">
+      <c r="R59" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="S50" s="22" t="inlineStr">
+      <c r="S59" s="22" t="inlineStr">
         <is>
           <t>Somehow Survives: the first hit that would knock him out leaves him at 1 HP instead.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="19" t="inlineStr">
+    <row r="60" s="16">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>Chachamaru</t>
         </is>
       </c>
-      <c r="B51" s="19" t="inlineStr">
+      <c r="B60" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C60" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D60" s="19" t="inlineStr">
         <is>
           <t>Tamayo's cat · back-pocket helper</t>
         </is>
       </c>
-      <c r="E51" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="20" t="n"/>
-      <c r="G51" s="20" t="n"/>
-      <c r="H51" s="20" t="n"/>
-      <c r="I51" s="20" t="n"/>
-      <c r="J51" s="20" t="n"/>
-      <c r="K51" s="21" t="n"/>
-      <c r="L51" s="21" t="n"/>
-      <c r="M51" s="20" t="n"/>
-      <c r="N51" s="20" t="n"/>
-      <c r="O51" s="21" t="n"/>
-      <c r="P51" s="19" t="inlineStr">
+      <c r="E60" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="20" t="n"/>
+      <c r="G60" s="20" t="n"/>
+      <c r="H60" s="20" t="n"/>
+      <c r="I60" s="20" t="n"/>
+      <c r="J60" s="20" t="n"/>
+      <c r="K60" s="21" t="n"/>
+      <c r="L60" s="21" t="n"/>
+      <c r="M60" s="20" t="n"/>
+      <c r="N60" s="20" t="n"/>
+      <c r="O60" s="21" t="n"/>
+      <c r="P60" s="19" t="inlineStr">
         <is>
           <t>Medicine Delivery</t>
         </is>
       </c>
-      <c r="Q51" s="22" t="inlineStr">
-        <is>
-          <t>Every fighter on your team heals half of their current health (50% becomes 75%).</t>
-        </is>
-      </c>
-      <c r="R51" s="20" t="n"/>
-      <c r="S51" s="22" t="inlineStr">
+      <c r="Q60" s="22" t="inlineStr">
+        <is>
+          <t>Your most hurt fighter heals half of their current health (50% becomes 75%).</t>
+        </is>
+      </c>
+      <c r="R60" s="20" t="n"/>
+      <c r="S60" s="22" t="inlineStr">
         <is>
           <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+    <row r="61" s="16">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>Hotaru Haganezuka</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Swordsmith · back-pocket helper</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="20" t="n"/>
+      <c r="G61" s="20" t="n"/>
+      <c r="H61" s="20" t="n"/>
+      <c r="I61" s="20" t="n"/>
+      <c r="J61" s="20" t="n"/>
+      <c r="K61" s="21" t="n"/>
+      <c r="L61" s="21" t="n"/>
+      <c r="M61" s="20" t="n"/>
+      <c r="N61" s="20" t="n"/>
+      <c r="O61" s="21" t="n"/>
+      <c r="P61" s="19" t="inlineStr">
+        <is>
+          <t>Reforged Blade</t>
+        </is>
+      </c>
+      <c r="Q61" s="22" t="inlineStr">
+        <is>
+          <t>Your fighter with the longest wait for their special gets it ready for next round.</t>
+        </is>
+      </c>
+      <c r="R61" s="20" t="n"/>
+      <c r="S61" s="22" t="inlineStr">
+        <is>
+          <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" s="16">
+      <c r="A62" s="19" t="inlineStr">
         <is>
           <t>Kasugai Crow</t>
         </is>
       </c>
-      <c r="B52" s="19" t="inlineStr">
+      <c r="B62" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="C52" s="19" t="inlineStr">
+      <c r="C62" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>Messenger crow · back-pocket helper</t>
         </is>
       </c>
-      <c r="E52" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="20" t="n"/>
-      <c r="G52" s="20" t="n"/>
-      <c r="H52" s="20" t="n"/>
-      <c r="I52" s="20" t="n"/>
-      <c r="J52" s="20" t="n"/>
-      <c r="K52" s="21" t="n"/>
-      <c r="L52" s="21" t="n"/>
-      <c r="M52" s="20" t="n"/>
-      <c r="N52" s="20" t="n"/>
-      <c r="O52" s="21" t="n"/>
-      <c r="P52" s="19" t="inlineStr">
+      <c r="E62" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="20" t="n"/>
+      <c r="G62" s="20" t="n"/>
+      <c r="H62" s="20" t="n"/>
+      <c r="I62" s="20" t="n"/>
+      <c r="J62" s="20" t="n"/>
+      <c r="K62" s="21" t="n"/>
+      <c r="L62" s="21" t="n"/>
+      <c r="M62" s="20" t="n"/>
+      <c r="N62" s="20" t="n"/>
+      <c r="O62" s="21" t="n"/>
+      <c r="P62" s="19" t="inlineStr">
         <is>
           <t>Scouting Report</t>
         </is>
       </c>
-      <c r="Q52" s="22" t="inlineStr">
+      <c r="Q62" s="22" t="inlineStr">
         <is>
           <t>After both sides lock in, the crow shows you the enemy's moves, and you can change yours before the round plays.</t>
         </is>
       </c>
-      <c r="R52" s="20" t="n"/>
-      <c r="S52" s="22" t="inlineStr">
+      <c r="R62" s="20" t="n"/>
+      <c r="S62" s="22" t="inlineStr">
         <is>
           <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+    <row r="63" s="16">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>Muscle Mice</t>
         </is>
       </c>
-      <c r="B53" s="19" t="inlineStr">
+      <c r="B63" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Helper</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>Tengen's mice · back-pocket helper</t>
         </is>
       </c>
-      <c r="E53" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="20" t="n"/>
-      <c r="G53" s="20" t="n"/>
-      <c r="H53" s="20" t="n"/>
-      <c r="I53" s="20" t="n"/>
-      <c r="J53" s="20" t="n"/>
-      <c r="K53" s="21" t="n"/>
-      <c r="L53" s="21" t="n"/>
-      <c r="M53" s="20" t="n"/>
-      <c r="N53" s="20" t="n"/>
-      <c r="O53" s="21" t="n"/>
-      <c r="P53" s="19" t="inlineStr">
+      <c r="E63" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="20" t="n"/>
+      <c r="G63" s="20" t="n"/>
+      <c r="H63" s="20" t="n"/>
+      <c r="I63" s="20" t="n"/>
+      <c r="J63" s="20" t="n"/>
+      <c r="K63" s="21" t="n"/>
+      <c r="L63" s="21" t="n"/>
+      <c r="M63" s="20" t="n"/>
+      <c r="N63" s="20" t="n"/>
+      <c r="O63" s="21" t="n"/>
+      <c r="P63" s="19" t="inlineStr">
         <is>
           <t>Flex!</t>
         </is>
       </c>
-      <c r="Q53" s="22" t="inlineStr">
+      <c r="Q63" s="22" t="inlineStr">
         <is>
           <t>Every fighter on your team gets +2 PWR for this round.</t>
         </is>
       </c>
-      <c r="R53" s="20" t="n"/>
-      <c r="S53" s="22" t="inlineStr">
+      <c r="R63" s="20" t="n"/>
+      <c r="S63" s="22" t="inlineStr">
         <is>
           <t>Back-pocket helper: no fighter slot, not on the battlefield, used once on a round you choose.</t>
         </is>
       </c>
     </row>
-    <row r="54"/>
-    <row r="55">
-      <c r="A55" s="24" t="inlineStr">
+    <row r="64"/>
+    <row r="65">
+      <c r="A65" s="24" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 25 2026). Black cells are formulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="25" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>Blue numbers are the game's current stats (from Squad Draft, Oct 26 2026). Black cells are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
         <is>
           <t>"1 HP = % of bar": how much of a fighter's bar one point of damage removes. Smaller = tankier.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="25" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
         <is>
           <t>Pink rows are Mark-awakened versions (+8 HP, +4 PWR, +2 SPD, +1 DEF, special 1 round faster; cost set per character). Gold rows are Legends.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Retired Tengen and Final-Form Muzan are second versions (one or the other is dealt). Helpers (1 pt) sit in the back pocket and have no fighting stats.</t>
+    <row r="69">
+      <c r="A69" s="25" t="inlineStr">
+        <is>
+          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Second versions share a character slot (one or the other is dealt): Retired Tengen, Final-Form Muzan, Demon King Tanjiro, Awakened Nezuko, Zohakuten. Helpers (1 pt) sit in the back pocket and have no fighting stats.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S53"/>
+  <autoFilter ref="A1:S63"/>
   <conditionalFormatting sqref="F2:F53">
     <cfRule type="dataBar" priority="1">
       <dataBar minLength="10" maxLength="90" showValue="1">
@@ -4427,6 +5148,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -4464,7 +5186,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="29">
-        <f>IF(A5="","",INDEX(Roster!$F$2:$F$53,MATCH(A5,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A5="","",INDEX(Roster!$F$2:$F$63,MATCH(A5,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D5" s="30">
@@ -4486,7 +5208,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="29">
-        <f>IF(A6="","",INDEX(Roster!$F$2:$F$53,MATCH(A6,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A6="","",INDEX(Roster!$F$2:$F$63,MATCH(A6,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D6" s="30">
@@ -4508,7 +5230,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="29">
-        <f>IF(A7="","",INDEX(Roster!$F$2:$F$53,MATCH(A7,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A7="","",INDEX(Roster!$F$2:$F$63,MATCH(A7,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D7" s="30">
@@ -4530,7 +5252,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="29">
-        <f>IF(A8="","",INDEX(Roster!$F$2:$F$53,MATCH(A8,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A8="","",INDEX(Roster!$F$2:$F$63,MATCH(A8,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D8" s="30">
@@ -4552,7 +5274,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="29">
-        <f>IF(A9="","",INDEX(Roster!$F$2:$F$53,MATCH(A9,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A9="","",INDEX(Roster!$F$2:$F$63,MATCH(A9,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D9" s="30">
@@ -4568,7 +5290,7 @@
       <c r="A10" s="28" t="n"/>
       <c r="B10" s="28" t="n"/>
       <c r="C10" s="29">
-        <f>IF(A10="","",INDEX(Roster!$F$2:$F$53,MATCH(A10,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A10="","",INDEX(Roster!$F$2:$F$63,MATCH(A10,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D10" s="30">
@@ -4584,7 +5306,7 @@
       <c r="A11" s="28" t="n"/>
       <c r="B11" s="28" t="n"/>
       <c r="C11" s="29">
-        <f>IF(A11="","",INDEX(Roster!$F$2:$F$53,MATCH(A11,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A11="","",INDEX(Roster!$F$2:$F$63,MATCH(A11,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D11" s="30">
@@ -4600,7 +5322,7 @@
       <c r="A12" s="28" t="n"/>
       <c r="B12" s="28" t="n"/>
       <c r="C12" s="29">
-        <f>IF(A12="","",INDEX(Roster!$F$2:$F$53,MATCH(A12,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A12="","",INDEX(Roster!$F$2:$F$63,MATCH(A12,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D12" s="30">
@@ -4616,7 +5338,7 @@
       <c r="A13" s="28" t="n"/>
       <c r="B13" s="28" t="n"/>
       <c r="C13" s="29">
-        <f>IF(A13="","",INDEX(Roster!$F$2:$F$53,MATCH(A13,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A13="","",INDEX(Roster!$F$2:$F$63,MATCH(A13,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D13" s="30">
@@ -4632,7 +5354,7 @@
       <c r="A14" s="28" t="n"/>
       <c r="B14" s="28" t="n"/>
       <c r="C14" s="29">
-        <f>IF(A14="","",INDEX(Roster!$F$2:$F$53,MATCH(A14,Roster!$A$2:$A$53,0)))</f>
+        <f>IF(A14="","",INDEX(Roster!$F$2:$F$63,MATCH(A14,Roster!$A$2:$A$63,0)))</f>
         <v/>
       </c>
       <c r="D14" s="30">
@@ -4644,6 +5366,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reprice Gyutaro (8 pts) and Daki (6 pts) so the pair is strong, not broken
Gyutaro 40/12/9/5, Daki 30/10/9/4. Canon checks pass: Tengen beats Daki, Daki beats Tanjiro,
Gyutaro beats Tengen, Tengen + Mark Tanjiro beat Gyutaro. Pair wins ~58% (was 71%).
Story Entertainment District: Gyutaro + Daki + Hand Demon, 17 pts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -1486,19 +1486,19 @@
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G13" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="H13" s="20" t="n">
-        <v>8</v>
-      </c>
       <c r="I13" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13" s="20" t="n">
         <v>2</v>
@@ -1634,19 +1634,19 @@
         </is>
       </c>
       <c r="E15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="I15" s="20" t="n">
         <v>4</v>
-      </c>
-      <c r="F15" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="G15" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="H15" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="I15" s="20" t="n">
-        <v>3</v>
       </c>
       <c r="J15" s="20" t="n">
         <v>2</v>
@@ -5066,7 +5066,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="24" t="inlineStr">
         <is>
@@ -5148,7 +5147,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -5366,7 +5364,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Hantengu: four emotions at once, merging into Zohakuten
When Hantengu falls, Sekido, Karaku, Aizetsu and Urogi all appear (smaller than before).
When the last emotion falls they merge into Zohakuten, who is no longer a separate card.
Tuned to ~55% at 20 pts (was 33%; the untuned chain won 92%).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -1316,19 +1316,19 @@
       </c>
       <c r="S10" s="22" t="inlineStr">
         <is>
-          <t>Splitting Emotions: when Hantengu falls he splits into Sekido and Karaku. When Sekido falls, Aizetsu takes his place; when Karaku falls, Urogi does. Beat all five to win.</t>
+          <t>Splitting Emotions: when Hantengu falls he splits into his four emotions: Sekido, Karaku, Aizetsu and Urogi. When the last of them falls, they merge into Zohakuten. Beat him too to win.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26.85" customHeight="1" s="16">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Zohakuten</t>
+          <t>Gyutaro</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Hatred</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1338,26 +1338,26 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 4 · Hatred</t>
+          <t>Upper Moon 6</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" s="20" t="n">
         <v>9</v>
       </c>
       <c r="I11" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J11" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" s="21">
         <f>1/F11</f>
@@ -1377,12 +1377,12 @@
       </c>
       <c r="P11" s="19" t="inlineStr">
         <is>
-          <t>Wood Dragons</t>
+          <t>Flying Blood Sickles</t>
         </is>
       </c>
       <c r="Q11" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−4, even through Defend.</t>
+          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
         </is>
       </c>
       <c r="R11" s="20" t="n">
@@ -1390,14 +1390,14 @@
       </c>
       <c r="S11" s="22" t="inlineStr">
         <is>
-          <t>Hantengu's Hatred: his emotions merged into one body. He doesn't split.</t>
+          <t>Two as One: with Daki on his team he gets +2 PWR. If one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each). Knock both out in the same round to stop it.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26.85" customHeight="1" s="16">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>Gyokko</t>
+          <t>Daki</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
@@ -1412,20 +1412,20 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 5</t>
+          <t>Upper Moon 6</t>
         </is>
       </c>
       <c r="E12" s="20" t="n">
         <v>6</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G12" s="20" t="n">
         <v>10</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I12" s="20" t="n">
         <v>4</v>
@@ -1451,23 +1451,27 @@
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>Water Prison Pot</t>
+          <t>Obi Sashes</t>
         </is>
       </c>
       <c r="Q12" s="22" t="inlineStr">
         <is>
-          <t>Traps one enemy: it takes PWR−2 (ignores DEF) and can't act next round.</t>
+          <t>Every enemy takes PWR−3.</t>
         </is>
       </c>
       <c r="R12" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S12" s="22" t="n"/>
+      <c r="S12" s="22" t="inlineStr">
+        <is>
+          <t>Two as One: with Gyutaro on her team, if one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each).</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26.85" customHeight="1" s="16">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Gyutaro</t>
+          <t>Gyokko</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -1482,23 +1486,23 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6</t>
+          <t>Upper Moon 5</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="F13" s="20" t="n">
-        <v>40</v>
-      </c>
-      <c r="G13" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>9</v>
-      </c>
       <c r="I13" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="20" t="n">
         <v>2</v>
@@ -1521,22 +1525,18 @@
       </c>
       <c r="P13" s="19" t="inlineStr">
         <is>
-          <t>Flying Blood Sickles</t>
+          <t>Water Prison Pot</t>
         </is>
       </c>
       <c r="Q13" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4 and is poisoned 2/round for 2 rounds.</t>
+          <t>Traps one enemy: it takes PWR−2 (ignores DEF) and can't act next round.</t>
         </is>
       </c>
       <c r="R13" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S13" s="22" t="inlineStr">
-        <is>
-          <t>Two as One: with Daki on his team he gets +2 PWR. If one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each). Knock both out in the same round to stop it.</t>
-        </is>
-      </c>
+      <c r="S13" s="22" t="n"/>
     </row>
     <row r="14" ht="26.85" customHeight="1" s="16">
       <c r="A14" s="19" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="15" ht="26.85" customHeight="1" s="16">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>Daki</t>
+          <t>Enmu</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
@@ -1630,26 +1630,26 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 6</t>
+          <t>Lower Moon 1</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I15" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J15" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15" s="21">
         <f>1/F15</f>
@@ -1669,27 +1669,23 @@
       </c>
       <c r="P15" s="19" t="inlineStr">
         <is>
-          <t>Obi Sashes</t>
+          <t>Forced Sleep</t>
         </is>
       </c>
       <c r="Q15" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes PWR−3.</t>
+          <t>Every enemy has to wait 2 more rounds for their special.</t>
         </is>
       </c>
       <c r="R15" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S15" s="22" t="inlineStr">
-        <is>
-          <t>Two as One: with Gyutaro on her team, if one of them falls while the other is still standing, they get back up at the end of the round with 30% health (once each).</t>
-        </is>
-      </c>
+      <c r="S15" s="22" t="n"/>
     </row>
     <row r="16" ht="26.85" customHeight="1" s="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>Enmu</t>
+          <t>Nakime</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
@@ -1704,26 +1700,26 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 1</t>
+          <t>Upper Moon 4 · Infinity Castle</t>
         </is>
       </c>
       <c r="E16" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G16" s="20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="21">
         <f>1/F16</f>
@@ -1743,23 +1739,27 @@
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Forced Sleep</t>
+          <t>Castle Shift</t>
         </is>
       </c>
       <c r="Q16" s="22" t="inlineStr">
         <is>
-          <t>Every enemy has to wait 2 more rounds for their special.</t>
+          <t>Moves first. Sends an enemy to another room: they can't act and can't be hit this round.</t>
         </is>
       </c>
       <c r="R16" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S16" s="22" t="n"/>
+      <c r="S16" s="22" t="inlineStr">
+        <is>
+          <t>Biwa, not blade: she never attacks. Her basic move, Biwa Strum, makes an enemy act last this round. If she's the last one standing on her team, she flees and counts as knocked out.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="26.85" customHeight="1" s="16">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Nakime</t>
+          <t>Rui</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
@@ -1774,26 +1774,26 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Upper Moon 4 · Infinity Castle</t>
+          <t>Lower Moon 5</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I17" s="20" t="n">
         <v>4</v>
       </c>
       <c r="J17" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="21">
         <f>1/F17</f>
@@ -1813,27 +1813,23 @@
       </c>
       <c r="P17" s="19" t="inlineStr">
         <is>
-          <t>Castle Shift</t>
+          <t>Cutting Thread Cage</t>
         </is>
       </c>
       <c r="Q17" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Sends an enemy to another room: they can't act and can't be hit this round.</t>
+          <t>Strike for PWR and stun the target next round.</t>
         </is>
       </c>
       <c r="R17" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S17" s="22" t="inlineStr">
-        <is>
-          <t>Biwa, not blade: she never attacks. Her basic move, Biwa Strum, makes an enemy act last this round. If she's the last one standing on her team, she flees and counts as knocked out.</t>
-        </is>
-      </c>
+      <c r="S17" s="22" t="n"/>
     </row>
     <row r="18" ht="26.85" customHeight="1" s="16">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Rui</t>
+          <t>Yahaba</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
@@ -1848,23 +1844,23 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Lower Moon 5</t>
+          <t>Arrow demon</t>
         </is>
       </c>
       <c r="E18" s="20" t="n">
         <v>4</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G18" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J18" s="20" t="n">
         <v>1</v>
@@ -1887,23 +1883,27 @@
       </c>
       <c r="P18" s="19" t="inlineStr">
         <is>
-          <t>Cutting Thread Cage</t>
+          <t>Vector Arrows</t>
         </is>
       </c>
       <c r="Q18" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR and stun the target next round.</t>
+          <t>Moves first. Bends an enemy's aim: every hit they throw this round misses.</t>
         </is>
       </c>
       <c r="R18" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="S18" s="22" t="n"/>
+      <c r="S18" s="22" t="inlineStr">
+        <is>
+          <t>Temari &amp; Arrows: with Susamaru on his team, his arrows guide her hits past Defend.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="26.85" customHeight="1" s="16">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Yahaba</t>
+          <t>Kyogai</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -1918,20 +1918,20 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Arrow demon</t>
+          <t>Former Lower Moon</t>
         </is>
       </c>
       <c r="E19" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" s="20" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G19" s="20" t="n">
         <v>6</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I19" s="20" t="n">
         <v>3</v>
@@ -1957,27 +1957,23 @@
       </c>
       <c r="P19" s="19" t="inlineStr">
         <is>
-          <t>Vector Arrows</t>
+          <t>Drum Room Spin</t>
         </is>
       </c>
       <c r="Q19" s="22" t="inlineStr">
         <is>
-          <t>Moves first. Bends an enemy's aim: every hit they throw this round misses.</t>
+          <t>Flip the room. The target is stunned next round.</t>
         </is>
       </c>
       <c r="R19" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S19" s="22" t="inlineStr">
-        <is>
-          <t>Temari &amp; Arrows: with Susamaru on his team, his arrows guide her hits past Defend.</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="S19" s="22" t="n"/>
     </row>
     <row r="20" ht="26.85" customHeight="1" s="16">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Kyogai</t>
+          <t>Susamaru</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
@@ -1992,7 +1988,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Former Lower Moon</t>
+          <t>Temari demon</t>
         </is>
       </c>
       <c r="E20" s="20" t="n">
@@ -2002,10 +1998,10 @@
         <v>22</v>
       </c>
       <c r="G20" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H20" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I20" s="20" t="n">
         <v>3</v>
@@ -2031,23 +2027,27 @@
       </c>
       <c r="P20" s="19" t="inlineStr">
         <is>
-          <t>Drum Room Spin</t>
+          <t>Temari Barrage</t>
         </is>
       </c>
       <c r="Q20" s="22" t="inlineStr">
         <is>
-          <t>Flip the room. The target is stunned next round.</t>
+          <t>Strike your target and one other enemy for PWR−1.</t>
         </is>
       </c>
       <c r="R20" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="S20" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S20" s="22" t="inlineStr">
+        <is>
+          <t>Temari &amp; Arrows: with Yahaba on her team, her hits slip past Defend.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="26.85" customHeight="1" s="16">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Susamaru</t>
+          <t>Swamp Demon</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
@@ -2062,23 +2062,23 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Temari demon</t>
+          <t>Lesser demon</t>
         </is>
       </c>
       <c r="E21" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F21" s="20" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G21" s="20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H21" s="20" t="n">
         <v>8</v>
       </c>
       <c r="I21" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" s="20" t="n">
         <v>1</v>
@@ -2101,27 +2101,23 @@
       </c>
       <c r="P21" s="19" t="inlineStr">
         <is>
-          <t>Temari Barrage</t>
+          <t>Swamp Dive</t>
         </is>
       </c>
       <c r="Q21" s="22" t="inlineStr">
         <is>
-          <t>Strike your target and one other enemy for PWR−1.</t>
+          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
         </is>
       </c>
       <c r="R21" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="S21" s="22" t="inlineStr">
-        <is>
-          <t>Temari &amp; Arrows: with Yahaba on her team, her hits slip past Defend.</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="S21" s="22" t="n"/>
     </row>
     <row r="22" ht="26.85" customHeight="1" s="16">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>Swamp Demon</t>
+          <t>Hand Demon</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
@@ -2136,23 +2132,23 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Lesser demon</t>
+          <t>Final Selection</t>
         </is>
       </c>
       <c r="E22" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I22" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J22" s="20" t="n">
         <v>1</v>
@@ -2175,12 +2171,12 @@
       </c>
       <c r="P22" s="19" t="inlineStr">
         <is>
-          <t>Swamp Dive</t>
+          <t>Grasping Arms</t>
         </is>
       </c>
       <c r="Q22" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Sinks out of reach this round and strikes for PWR+1.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R22" s="20" t="n">
@@ -2191,12 +2187,12 @@
     <row r="23" ht="26.85" customHeight="1" s="16">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Hand Demon</t>
+          <t>Aizetsu (Sorrow)</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Split form</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
@@ -2206,20 +2202,20 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Final Selection</t>
+          <t>Hantengu split · Sorrow</t>
         </is>
       </c>
       <c r="E23" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23" s="20" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G23" s="20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H23" s="20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I23" s="20" t="n">
         <v>3</v>
@@ -2245,23 +2241,27 @@
       </c>
       <c r="P23" s="19" t="inlineStr">
         <is>
-          <t>Grasping Arms</t>
+          <t>Cross Spear</t>
         </is>
       </c>
       <c r="Q23" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Strike for PWR+4.</t>
         </is>
       </c>
       <c r="R23" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="S23" s="22" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="S23" s="22" t="inlineStr">
+        <is>
+          <t>Appears when Hantengu falls (with all four emotions).</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="26.85" customHeight="1" s="16">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Aizetsu (Sorrow)</t>
+          <t>Karaku (Joy)</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -2276,20 +2276,20 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Sorrow</t>
+          <t>Hantengu split · Joy</t>
         </is>
       </c>
       <c r="E24" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G24" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H24" s="20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I24" s="20" t="n">
         <v>3</v>
@@ -2315,27 +2315,27 @@
       </c>
       <c r="P24" s="19" t="inlineStr">
         <is>
-          <t>Cross Spear</t>
+          <t>Gale Fan</t>
         </is>
       </c>
       <c r="Q24" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+4.</t>
+          <t>Strike for PWR+3.</t>
         </is>
       </c>
       <c r="R24" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S24" s="22" t="inlineStr">
         <is>
-          <t>Appears when Sekido falls. Not drafted.</t>
+          <t>Appears when Hantengu falls (with all four emotions).</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26.85" customHeight="1" s="16">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Karaku (Joy)</t>
+          <t>Sekido (Anger)</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
@@ -2350,20 +2350,20 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Joy</t>
+          <t>Hantengu split · Anger</t>
         </is>
       </c>
       <c r="E25" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="20" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G25" s="20" t="n">
         <v>7</v>
       </c>
       <c r="H25" s="20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I25" s="20" t="n">
         <v>3</v>
@@ -2389,27 +2389,27 @@
       </c>
       <c r="P25" s="19" t="inlineStr">
         <is>
-          <t>Gale Fan</t>
+          <t>Lightning Staff</t>
         </is>
       </c>
       <c r="Q25" s="22" t="inlineStr">
         <is>
-          <t>Strike for PWR+3.</t>
+          <t>Every enemy takes 4, ignores DEF.</t>
         </is>
       </c>
       <c r="R25" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S25" s="22" t="inlineStr">
         <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
+          <t>Appears when Hantengu falls (with all four emotions).</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26.85" customHeight="1" s="16">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Sekido (Anger)</t>
+          <t>Urogi (Pleasure)</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
@@ -2424,23 +2424,23 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Anger</t>
+          <t>Hantengu split · Pleasure</t>
         </is>
       </c>
       <c r="E26" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I26" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" s="20" t="n">
         <v>1</v>
@@ -2463,27 +2463,27 @@
       </c>
       <c r="P26" s="19" t="inlineStr">
         <is>
-          <t>Lightning Staff</t>
+          <t>Sky Dive</t>
         </is>
       </c>
       <c r="Q26" s="22" t="inlineStr">
         <is>
-          <t>Every enemy takes 4, ignores DEF.</t>
+          <t>Moves early. Swoops down for PWR+2.</t>
         </is>
       </c>
       <c r="R26" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S26" s="22" t="inlineStr">
         <is>
-          <t>Appears when Hantengu falls. Not drafted.</t>
+          <t>Appears when Hantengu falls (with all four emotions).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26.85" customHeight="1" s="16">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>Urogi (Pleasure)</t>
+          <t>Zohakuten (Hatred)</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
@@ -2498,26 +2498,26 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Hantengu split · Pleasure</t>
+          <t>Hantengu merged · Hatred</t>
         </is>
       </c>
       <c r="E27" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="G27" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="G27" s="20" t="n">
-        <v>6</v>
-      </c>
       <c r="H27" s="20" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I27" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J27" s="20" t="n">
         <v>2</v>
-      </c>
-      <c r="J27" s="20" t="n">
-        <v>1</v>
       </c>
       <c r="K27" s="21">
         <f>1/F27</f>
@@ -2537,20 +2537,20 @@
       </c>
       <c r="P27" s="19" t="inlineStr">
         <is>
-          <t>Sky Dive</t>
+          <t>Wood Dragons</t>
         </is>
       </c>
       <c r="Q27" s="22" t="inlineStr">
         <is>
-          <t>Moves early. Swoops down for PWR+2.</t>
+          <t>Every enemy takes PWR−4, even through Defend.</t>
         </is>
       </c>
       <c r="R27" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S27" s="22" t="inlineStr">
         <is>
-          <t>Appears when Karaku falls. Not drafted.</t>
+          <t>Appears when the last of the four emotions falls: they merge into him.</t>
         </is>
       </c>
     </row>
@@ -5066,6 +5066,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="24" t="inlineStr">
         <is>
@@ -5097,7 +5098,7 @@
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
         <is>
-          <t>Split forms (cost 0) are never drafted: they join Hantengu's team when he or another form falls. Second versions share a character slot (one or the other is dealt): Retired Tengen, Final-Form Muzan, Demon King Tanjiro, Awakened Nezuko, Zohakuten. Helpers (1 pt) sit in the back pocket and have no fighting stats.</t>
+          <t>Split forms (cost 0) are never drafted: when Hantengu falls his four emotions appear, and when the last of them falls they merge into Zohakuten. Second versions share a character slot (one or the other is dealt): Retired Tengen, Final-Form Muzan, Demon King Tanjiro, Awakened Nezuko. Helpers (1 pt) sit in the back pocket and have no fighting stats.</t>
         </is>
       </c>
     </row>
@@ -5147,6 +5148,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -5364,6 +5366,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Old Yoriichi and Demon King Tanjiro cost 17 pts, with stats to match
Old Yoriichi 50 HP / 14 PWR (~55%), Demon King Tanjiro 54 HP / 18 PWR (~62%).
Story: flashback boosts Kokushibo +4 PWR; Demon King finale +15% HP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad-Draft-Character-Stats.xlsx
+++ b/Squad-Draft-Character-Stats.xlsx
@@ -764,13 +764,13 @@
         </is>
       </c>
       <c r="E3" s="20" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3" s="20" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G3" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H3" s="20" t="n">
         <v>11</v>
@@ -1054,13 +1054,13 @@
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" s="20" t="n">
         <v>11</v>
@@ -5066,7 +5066,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="24" t="inlineStr">
         <is>
@@ -5148,7 +5147,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -5366,7 +5364,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="16">
       <c r="A16" s="25" t="inlineStr">
         <is>

</xml_diff>